<commit_message>
saida: ISAIAS taxa de serviço em uma aba por loja
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015XeuzNyreGoe8Jd1wBUgeX
</commit_message>
<xml_diff>
--- a/saida/isaias_taxa_servico_2026-10-01_a_18.xlsx
+++ b/saida/isaias_taxa_servico_2026-10-01_a_18.xlsx
@@ -7,7 +7,8 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cupons sem taxa cobrados na máq" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ISAIAS 01" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ISAIAS 02" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,10 +414,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P89"/>
+  <dimension ref="A1:P83"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="21" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
@@ -542,10 +543,8 @@
           <t>18:11</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>42804</t>
-        </is>
+      <c r="F2" t="n">
+        <v>42804</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -562,10 +561,8 @@
           <t>JOSE HENRIQUE ROSA</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>14</t>
-        </is>
+      <c r="J2" t="n">
+        <v>14</v>
       </c>
       <c r="K2" t="n">
         <v>269</v>
@@ -618,10 +615,8 @@
           <t>20:11</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>42817</t>
-        </is>
+      <c r="F3" t="n">
+        <v>42817</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
@@ -638,10 +633,8 @@
           <t>MATEUS AUGUSTO NASCIMENTO COSTA</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>30</t>
-        </is>
+      <c r="J3" t="n">
+        <v>30</v>
       </c>
       <c r="K3" t="n">
         <v>160</v>
@@ -694,10 +687,8 @@
           <t>21:06</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>42818</t>
-        </is>
+      <c r="F4" t="n">
+        <v>42818</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
@@ -714,10 +705,8 @@
           <t>MATEUS AUGUSTO NASCIMENTO COSTA</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>29</t>
-        </is>
+      <c r="J4" t="n">
+        <v>29</v>
       </c>
       <c r="K4" t="n">
         <v>244</v>
@@ -770,10 +759,8 @@
           <t>21:24</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>42823</t>
-        </is>
+      <c r="F5" t="n">
+        <v>42823</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
@@ -790,10 +777,8 @@
           <t>CAIO VINICIUS DOS SANTOS SILVA</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>30</t>
-        </is>
+      <c r="J5" t="n">
+        <v>30</v>
       </c>
       <c r="K5" t="n">
         <v>88</v>
@@ -846,10 +831,8 @@
           <t>20:33</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>42877</t>
-        </is>
+      <c r="F6" t="n">
+        <v>42877</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
@@ -866,10 +849,8 @@
           <t>KEROLAINY LAWANY RIO BRANCO</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
+      <c r="J6" t="n">
+        <v>7</v>
       </c>
       <c r="K6" t="n">
         <v>151</v>
@@ -922,10 +903,8 @@
           <t>21:15</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>42879</t>
-        </is>
+      <c r="F7" t="n">
+        <v>42879</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
@@ -942,10 +921,8 @@
           <t>LUCAS DE MUSSI PALMA</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+      <c r="J7" t="n">
+        <v>3</v>
       </c>
       <c r="K7" t="n">
         <v>213.5</v>
@@ -998,10 +975,8 @@
           <t>21:31</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>42884</t>
-        </is>
+      <c r="F8" t="n">
+        <v>42884</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
@@ -1018,10 +993,8 @@
           <t>KEROLAINY LAWANY RIO BRANCO</t>
         </is>
       </c>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t>30</t>
-        </is>
+      <c r="J8" t="n">
+        <v>30</v>
       </c>
       <c r="K8" t="n">
         <v>168.5</v>
@@ -1074,10 +1047,8 @@
           <t>21:43</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>42887</t>
-        </is>
+      <c r="F9" t="n">
+        <v>42887</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
@@ -1094,10 +1065,8 @@
           <t>KEROLAINY LAWANY RIO BRANCO</t>
         </is>
       </c>
-      <c r="J9" t="inlineStr">
-        <is>
-          <t>26</t>
-        </is>
+      <c r="J9" t="n">
+        <v>26</v>
       </c>
       <c r="K9" t="n">
         <v>107.5</v>
@@ -1150,10 +1119,8 @@
           <t>21:58</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>42891</t>
-        </is>
+      <c r="F10" t="n">
+        <v>42891</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
@@ -1170,10 +1137,8 @@
           <t>DAVID FERNANDES DA CRUZ</t>
         </is>
       </c>
-      <c r="J10" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
+      <c r="J10" t="n">
+        <v>5</v>
       </c>
       <c r="K10" t="n">
         <v>150</v>
@@ -1226,10 +1191,8 @@
           <t>21:59</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>42892</t>
-        </is>
+      <c r="F11" t="n">
+        <v>42892</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
@@ -1246,10 +1209,8 @@
           <t>DAVID FERNANDES DA CRUZ</t>
         </is>
       </c>
-      <c r="J11" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
+      <c r="J11" t="n">
+        <v>7</v>
       </c>
       <c r="K11" t="n">
         <v>136.5</v>
@@ -1302,10 +1263,8 @@
           <t>22:03</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>42895</t>
-        </is>
+      <c r="F12" t="n">
+        <v>42895</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
@@ -1322,10 +1281,8 @@
           <t xml:space="preserve">DAIANA APARECIDA DOS SANTOS SILVA ALVES </t>
         </is>
       </c>
-      <c r="J12" t="inlineStr">
-        <is>
-          <t>252</t>
-        </is>
+      <c r="J12" t="n">
+        <v>252</v>
       </c>
       <c r="K12" t="n">
         <v>277</v>
@@ -1378,10 +1335,8 @@
           <t>22:06</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>42897</t>
-        </is>
+      <c r="F13" t="n">
+        <v>42897</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
@@ -1398,10 +1353,8 @@
           <t>KEROLAINY LAWANY RIO BRANCO</t>
         </is>
       </c>
-      <c r="J13" t="inlineStr">
-        <is>
-          <t>152</t>
-        </is>
+      <c r="J13" t="n">
+        <v>152</v>
       </c>
       <c r="K13" t="n">
         <v>104</v>
@@ -1454,10 +1407,8 @@
           <t>22:28</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>42902</t>
-        </is>
+      <c r="F14" t="n">
+        <v>42902</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
@@ -1474,10 +1425,8 @@
           <t xml:space="preserve">DAIANA APARECIDA DOS SANTOS SILVA ALVES </t>
         </is>
       </c>
-      <c r="J14" t="inlineStr">
-        <is>
-          <t>29</t>
-        </is>
+      <c r="J14" t="n">
+        <v>29</v>
       </c>
       <c r="K14" t="n">
         <v>213</v>
@@ -1530,10 +1479,8 @@
           <t>22:40</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>42908</t>
-        </is>
+      <c r="F15" t="n">
+        <v>42908</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
@@ -1550,10 +1497,8 @@
           <t xml:space="preserve">DAIANA APARECIDA DOS SANTOS SILVA ALVES </t>
         </is>
       </c>
-      <c r="J15" t="inlineStr">
-        <is>
-          <t>244</t>
-        </is>
+      <c r="J15" t="n">
+        <v>244</v>
       </c>
       <c r="K15" t="n">
         <v>517</v>
@@ -1606,10 +1551,8 @@
           <t>23:24</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>42921</t>
-        </is>
+      <c r="F16" t="n">
+        <v>42921</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
@@ -1626,10 +1569,8 @@
           <t xml:space="preserve">DANIEL BACELAR XAVIER </t>
         </is>
       </c>
-      <c r="J16" t="inlineStr">
-        <is>
-          <t>18</t>
-        </is>
+      <c r="J16" t="n">
+        <v>18</v>
       </c>
       <c r="K16" t="n">
         <v>149.5</v>
@@ -1682,10 +1623,8 @@
           <t>21:20</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>42983</t>
-        </is>
+      <c r="F17" t="n">
+        <v>42983</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
@@ -1702,10 +1641,8 @@
           <t xml:space="preserve">DANIEL BACELAR XAVIER </t>
         </is>
       </c>
-      <c r="J17" t="inlineStr">
-        <is>
-          <t>266</t>
-        </is>
+      <c r="J17" t="n">
+        <v>266</v>
       </c>
       <c r="K17" t="n">
         <v>135.5</v>
@@ -1758,10 +1695,8 @@
           <t>22:16</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>43013</t>
-        </is>
+      <c r="F18" t="n">
+        <v>43013</v>
       </c>
       <c r="G18" t="inlineStr">
         <is>
@@ -1778,10 +1713,8 @@
           <t>CAIO VINICIUS DOS SANTOS SILVA</t>
         </is>
       </c>
-      <c r="J18" t="inlineStr">
-        <is>
-          <t>28</t>
-        </is>
+      <c r="J18" t="n">
+        <v>28</v>
       </c>
       <c r="K18" t="n">
         <v>87</v>
@@ -1834,10 +1767,8 @@
           <t>23:25</t>
         </is>
       </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>43068</t>
-        </is>
+      <c r="F19" t="n">
+        <v>43068</v>
       </c>
       <c r="G19" t="inlineStr">
         <is>
@@ -1854,10 +1785,8 @@
           <t xml:space="preserve">DANIEL BACELAR XAVIER </t>
         </is>
       </c>
-      <c r="J19" t="inlineStr">
-        <is>
-          <t>208</t>
-        </is>
+      <c r="J19" t="n">
+        <v>208</v>
       </c>
       <c r="K19" t="n">
         <v>49</v>
@@ -1910,10 +1839,8 @@
           <t>23:26</t>
         </is>
       </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>43070</t>
-        </is>
+      <c r="F20" t="n">
+        <v>43070</v>
       </c>
       <c r="G20" t="inlineStr">
         <is>
@@ -1930,10 +1857,8 @@
           <t xml:space="preserve">DANIEL BACELAR XAVIER </t>
         </is>
       </c>
-      <c r="J20" t="inlineStr">
-        <is>
-          <t>185</t>
-        </is>
+      <c r="J20" t="n">
+        <v>185</v>
       </c>
       <c r="K20" t="n">
         <v>61</v>
@@ -1986,10 +1911,8 @@
           <t>23:30</t>
         </is>
       </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>43076</t>
-        </is>
+      <c r="F21" t="n">
+        <v>43076</v>
       </c>
       <c r="G21" t="inlineStr">
         <is>
@@ -2006,10 +1929,8 @@
           <t>MATEUS AUGUSTO NASCIMENTO COSTA</t>
         </is>
       </c>
-      <c r="J21" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
+      <c r="J21" t="n">
+        <v>6</v>
       </c>
       <c r="K21" t="n">
         <v>226</v>
@@ -2062,10 +1983,8 @@
           <t>23:30</t>
         </is>
       </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>43075</t>
-        </is>
+      <c r="F22" t="n">
+        <v>43075</v>
       </c>
       <c r="G22" t="inlineStr">
         <is>
@@ -2082,10 +2001,8 @@
           <t>MATEUS AUGUSTO NASCIMENTO COSTA</t>
         </is>
       </c>
-      <c r="J22" t="inlineStr">
-        <is>
-          <t>12</t>
-        </is>
+      <c r="J22" t="n">
+        <v>12</v>
       </c>
       <c r="K22" t="n">
         <v>148</v>
@@ -2138,10 +2055,8 @@
           <t>23:31</t>
         </is>
       </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>43078</t>
-        </is>
+      <c r="F23" t="n">
+        <v>43078</v>
       </c>
       <c r="G23" t="inlineStr">
         <is>
@@ -2158,10 +2073,8 @@
           <t>MATEUS AUGUSTO NASCIMENTO COSTA</t>
         </is>
       </c>
-      <c r="J23" t="inlineStr">
-        <is>
-          <t>17</t>
-        </is>
+      <c r="J23" t="n">
+        <v>17</v>
       </c>
       <c r="K23" t="n">
         <v>147.5</v>
@@ -2214,10 +2127,8 @@
           <t>23:45</t>
         </is>
       </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>43085</t>
-        </is>
+      <c r="F24" t="n">
+        <v>43085</v>
       </c>
       <c r="G24" t="inlineStr">
         <is>
@@ -2234,10 +2145,8 @@
           <t>DAVID FERNANDES DA CRUZ</t>
         </is>
       </c>
-      <c r="J24" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+      <c r="J24" t="n">
+        <v>3</v>
       </c>
       <c r="K24" t="n">
         <v>196.5</v>
@@ -2290,10 +2199,8 @@
           <t>20:28</t>
         </is>
       </c>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t>43117</t>
-        </is>
+      <c r="F25" t="n">
+        <v>43117</v>
       </c>
       <c r="G25" t="inlineStr">
         <is>
@@ -2310,10 +2217,8 @@
           <t>MATEUS AUGUSTO NASCIMENTO COSTA</t>
         </is>
       </c>
-      <c r="J25" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
+      <c r="J25" t="n">
+        <v>7</v>
       </c>
       <c r="K25" t="n">
         <v>124</v>
@@ -2366,10 +2271,8 @@
           <t>22:07</t>
         </is>
       </c>
-      <c r="F26" t="inlineStr">
-        <is>
-          <t>43138</t>
-        </is>
+      <c r="F26" t="n">
+        <v>43138</v>
       </c>
       <c r="G26" t="inlineStr">
         <is>
@@ -2386,10 +2289,8 @@
           <t>KEROLAINY LAWANY RIO BRANCO</t>
         </is>
       </c>
-      <c r="J26" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
+      <c r="J26" t="n">
+        <v>6</v>
       </c>
       <c r="K26" t="n">
         <v>94</v>
@@ -2442,10 +2343,8 @@
           <t>22:30</t>
         </is>
       </c>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>43151</t>
-        </is>
+      <c r="F27" t="n">
+        <v>43151</v>
       </c>
       <c r="G27" t="inlineStr">
         <is>
@@ -2462,10 +2361,8 @@
           <t>DAVID FERNANDES DA CRUZ</t>
         </is>
       </c>
-      <c r="J27" t="inlineStr">
-        <is>
-          <t>31</t>
-        </is>
+      <c r="J27" t="n">
+        <v>31</v>
       </c>
       <c r="K27" t="n">
         <v>105</v>
@@ -2518,10 +2415,8 @@
           <t>22:31</t>
         </is>
       </c>
-      <c r="F28" t="inlineStr">
-        <is>
-          <t>43153</t>
-        </is>
+      <c r="F28" t="n">
+        <v>43153</v>
       </c>
       <c r="G28" t="inlineStr">
         <is>
@@ -2538,10 +2433,8 @@
           <t>CAIO VINICIUS DOS SANTOS SILVA</t>
         </is>
       </c>
-      <c r="J28" t="inlineStr">
-        <is>
-          <t>179</t>
-        </is>
+      <c r="J28" t="n">
+        <v>179</v>
       </c>
       <c r="K28" t="n">
         <v>144</v>
@@ -2594,10 +2487,8 @@
           <t>12:55</t>
         </is>
       </c>
-      <c r="F29" t="inlineStr">
-        <is>
-          <t>43179</t>
-        </is>
+      <c r="F29" t="n">
+        <v>43179</v>
       </c>
       <c r="G29" t="inlineStr">
         <is>
@@ -2614,10 +2505,8 @@
           <t>CAIO VINICIUS DOS SANTOS SILVA</t>
         </is>
       </c>
-      <c r="J29" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
+      <c r="J29" t="n">
+        <v>11</v>
       </c>
       <c r="K29" t="n">
         <v>84</v>
@@ -2670,10 +2559,8 @@
           <t>18:52</t>
         </is>
       </c>
-      <c r="F30" t="inlineStr">
-        <is>
-          <t>43212</t>
-        </is>
+      <c r="F30" t="n">
+        <v>43212</v>
       </c>
       <c r="G30" t="inlineStr">
         <is>
@@ -2690,10 +2577,8 @@
           <t>JOSE HENRIQUE ROSA</t>
         </is>
       </c>
-      <c r="J30" t="inlineStr">
-        <is>
-          <t>15</t>
-        </is>
+      <c r="J30" t="n">
+        <v>15</v>
       </c>
       <c r="K30" t="n">
         <v>113</v>
@@ -2746,10 +2631,8 @@
           <t>21:16</t>
         </is>
       </c>
-      <c r="F31" t="inlineStr">
-        <is>
-          <t>43219</t>
-        </is>
+      <c r="F31" t="n">
+        <v>43219</v>
       </c>
       <c r="G31" t="inlineStr">
         <is>
@@ -2766,10 +2649,8 @@
           <t xml:space="preserve">DAIANA APARECIDA DOS SANTOS SILVA ALVES </t>
         </is>
       </c>
-      <c r="J31" t="inlineStr">
-        <is>
-          <t>29</t>
-        </is>
+      <c r="J31" t="n">
+        <v>29</v>
       </c>
       <c r="K31" t="n">
         <v>127</v>
@@ -2822,10 +2703,8 @@
           <t>21:24</t>
         </is>
       </c>
-      <c r="F32" t="inlineStr">
-        <is>
-          <t>43222</t>
-        </is>
+      <c r="F32" t="n">
+        <v>43222</v>
       </c>
       <c r="G32" t="inlineStr">
         <is>
@@ -2842,10 +2721,8 @@
           <t xml:space="preserve">DAIANA APARECIDA DOS SANTOS SILVA ALVES </t>
         </is>
       </c>
-      <c r="J32" t="inlineStr">
-        <is>
-          <t>157</t>
-        </is>
+      <c r="J32" t="n">
+        <v>157</v>
       </c>
       <c r="K32" t="n">
         <v>50</v>
@@ -2898,10 +2775,8 @@
           <t>22:26</t>
         </is>
       </c>
-      <c r="F33" t="inlineStr">
-        <is>
-          <t>43316</t>
-        </is>
+      <c r="F33" t="n">
+        <v>43316</v>
       </c>
       <c r="G33" t="inlineStr">
         <is>
@@ -2918,10 +2793,8 @@
           <t xml:space="preserve">DANIEL BACELAR XAVIER </t>
         </is>
       </c>
-      <c r="J33" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
+      <c r="J33" t="n">
+        <v>6</v>
       </c>
       <c r="K33" t="n">
         <v>143.5</v>
@@ -2974,10 +2847,8 @@
           <t>22:56</t>
         </is>
       </c>
-      <c r="F34" t="inlineStr">
-        <is>
-          <t>43322</t>
-        </is>
+      <c r="F34" t="n">
+        <v>43322</v>
       </c>
       <c r="G34" t="inlineStr">
         <is>
@@ -2994,10 +2865,8 @@
           <t>DAVID FERNANDES DA CRUZ</t>
         </is>
       </c>
-      <c r="J34" t="inlineStr">
-        <is>
-          <t>30</t>
-        </is>
+      <c r="J34" t="n">
+        <v>30</v>
       </c>
       <c r="K34" t="n">
         <v>93</v>
@@ -3050,10 +2919,8 @@
           <t>20:42</t>
         </is>
       </c>
-      <c r="F35" t="inlineStr">
-        <is>
-          <t>43366</t>
-        </is>
+      <c r="F35" t="n">
+        <v>43366</v>
       </c>
       <c r="G35" t="inlineStr">
         <is>
@@ -3070,10 +2937,8 @@
           <t>MATEUS AUGUSTO NASCIMENTO COSTA</t>
         </is>
       </c>
-      <c r="J35" t="inlineStr">
-        <is>
-          <t>29</t>
-        </is>
+      <c r="J35" t="n">
+        <v>29</v>
       </c>
       <c r="K35" t="n">
         <v>110.5</v>
@@ -3126,10 +2991,8 @@
           <t>21:17</t>
         </is>
       </c>
-      <c r="F36" t="inlineStr">
-        <is>
-          <t>43370</t>
-        </is>
+      <c r="F36" t="n">
+        <v>43370</v>
       </c>
       <c r="G36" t="inlineStr">
         <is>
@@ -3146,10 +3009,8 @@
           <t xml:space="preserve">DAIANA APARECIDA DOS SANTOS SILVA ALVES </t>
         </is>
       </c>
-      <c r="J36" t="inlineStr">
-        <is>
-          <t>14</t>
-        </is>
+      <c r="J36" t="n">
+        <v>14</v>
       </c>
       <c r="K36" t="n">
         <v>124.5</v>
@@ -3202,10 +3063,8 @@
           <t>21:24</t>
         </is>
       </c>
-      <c r="F37" t="inlineStr">
-        <is>
-          <t>43372</t>
-        </is>
+      <c r="F37" t="n">
+        <v>43372</v>
       </c>
       <c r="G37" t="inlineStr">
         <is>
@@ -3222,10 +3081,8 @@
           <t xml:space="preserve">DAIANA APARECIDA DOS SANTOS SILVA ALVES </t>
         </is>
       </c>
-      <c r="J37" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
+      <c r="J37" t="n">
+        <v>7</v>
       </c>
       <c r="K37" t="n">
         <v>159</v>
@@ -3278,10 +3135,8 @@
           <t>21:45</t>
         </is>
       </c>
-      <c r="F38" t="inlineStr">
-        <is>
-          <t>43379</t>
-        </is>
+      <c r="F38" t="n">
+        <v>43379</v>
       </c>
       <c r="G38" t="inlineStr">
         <is>
@@ -3298,10 +3153,8 @@
           <t xml:space="preserve">DAIANA APARECIDA DOS SANTOS SILVA ALVES </t>
         </is>
       </c>
-      <c r="J38" t="inlineStr">
-        <is>
-          <t>28</t>
-        </is>
+      <c r="J38" t="n">
+        <v>28</v>
       </c>
       <c r="K38" t="n">
         <v>191.5</v>
@@ -3354,10 +3207,8 @@
           <t>21:53</t>
         </is>
       </c>
-      <c r="F39" t="inlineStr">
-        <is>
-          <t>43382</t>
-        </is>
+      <c r="F39" t="n">
+        <v>43382</v>
       </c>
       <c r="G39" t="inlineStr">
         <is>
@@ -3374,10 +3225,8 @@
           <t>KEROLAINY LAWANY RIO BRANCO</t>
         </is>
       </c>
-      <c r="J39" t="inlineStr">
-        <is>
-          <t>31</t>
-        </is>
+      <c r="J39" t="n">
+        <v>31</v>
       </c>
       <c r="K39" t="n">
         <v>153</v>
@@ -3430,10 +3279,8 @@
           <t>23:09</t>
         </is>
       </c>
-      <c r="F40" t="inlineStr">
-        <is>
-          <t>43416</t>
-        </is>
+      <c r="F40" t="n">
+        <v>43416</v>
       </c>
       <c r="G40" t="inlineStr">
         <is>
@@ -3450,10 +3297,8 @@
           <t>KEROLAINY LAWANY RIO BRANCO</t>
         </is>
       </c>
-      <c r="J40" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
+      <c r="J40" t="n">
+        <v>7</v>
       </c>
       <c r="K40" t="n">
         <v>208</v>
@@ -3506,10 +3351,8 @@
           <t>20:11</t>
         </is>
       </c>
-      <c r="F41" t="inlineStr">
-        <is>
-          <t>43440</t>
-        </is>
+      <c r="F41" t="n">
+        <v>43440</v>
       </c>
       <c r="G41" t="inlineStr">
         <is>
@@ -3526,10 +3369,8 @@
           <t xml:space="preserve">DANIEL BACELAR XAVIER </t>
         </is>
       </c>
-      <c r="J41" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
+      <c r="J41" t="n">
+        <v>11</v>
       </c>
       <c r="K41" t="n">
         <v>215</v>
@@ -3582,10 +3423,8 @@
           <t>20:42</t>
         </is>
       </c>
-      <c r="F42" t="inlineStr">
-        <is>
-          <t>43444</t>
-        </is>
+      <c r="F42" t="n">
+        <v>43444</v>
       </c>
       <c r="G42" t="inlineStr">
         <is>
@@ -3602,10 +3441,8 @@
           <t xml:space="preserve">DANIEL BACELAR XAVIER </t>
         </is>
       </c>
-      <c r="J42" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
+      <c r="J42" t="n">
+        <v>6</v>
       </c>
       <c r="K42" t="n">
         <v>226</v>
@@ -3658,10 +3495,8 @@
           <t>21:15</t>
         </is>
       </c>
-      <c r="F43" t="inlineStr">
-        <is>
-          <t>43452</t>
-        </is>
+      <c r="F43" t="n">
+        <v>43452</v>
       </c>
       <c r="G43" t="inlineStr">
         <is>
@@ -3678,10 +3513,8 @@
           <t>LUCAS DE MUSSI PALMA</t>
         </is>
       </c>
-      <c r="J43" t="inlineStr">
-        <is>
-          <t>240</t>
-        </is>
+      <c r="J43" t="n">
+        <v>240</v>
       </c>
       <c r="K43" t="n">
         <v>257</v>
@@ -3734,10 +3567,8 @@
           <t>21:16</t>
         </is>
       </c>
-      <c r="F44" t="inlineStr">
-        <is>
-          <t>43454</t>
-        </is>
+      <c r="F44" t="n">
+        <v>43454</v>
       </c>
       <c r="G44" t="inlineStr">
         <is>
@@ -3754,10 +3585,8 @@
           <t xml:space="preserve">DANIEL BACELAR XAVIER </t>
         </is>
       </c>
-      <c r="J44" t="inlineStr">
-        <is>
-          <t>124</t>
-        </is>
+      <c r="J44" t="n">
+        <v>124</v>
       </c>
       <c r="K44" t="n">
         <v>52</v>
@@ -3810,10 +3639,8 @@
           <t>21:18</t>
         </is>
       </c>
-      <c r="F45" t="inlineStr">
-        <is>
-          <t>43456</t>
-        </is>
+      <c r="F45" t="n">
+        <v>43456</v>
       </c>
       <c r="G45" t="inlineStr">
         <is>
@@ -3830,10 +3657,8 @@
           <t xml:space="preserve">DANIEL BACELAR XAVIER </t>
         </is>
       </c>
-      <c r="J45" t="inlineStr">
-        <is>
-          <t>206</t>
-        </is>
+      <c r="J45" t="n">
+        <v>206</v>
       </c>
       <c r="K45" t="n">
         <v>256</v>
@@ -3886,10 +3711,8 @@
           <t>21:18</t>
         </is>
       </c>
-      <c r="F46" t="inlineStr">
-        <is>
-          <t>43457</t>
-        </is>
+      <c r="F46" t="n">
+        <v>43457</v>
       </c>
       <c r="G46" t="inlineStr">
         <is>
@@ -3906,10 +3729,8 @@
           <t xml:space="preserve">DANIEL BACELAR XAVIER </t>
         </is>
       </c>
-      <c r="J46" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
+      <c r="J46" t="n">
+        <v>7</v>
       </c>
       <c r="K46" t="n">
         <v>282</v>
@@ -3962,10 +3783,8 @@
           <t>21:18</t>
         </is>
       </c>
-      <c r="F47" t="inlineStr">
-        <is>
-          <t>43458</t>
-        </is>
+      <c r="F47" t="n">
+        <v>43458</v>
       </c>
       <c r="G47" t="inlineStr">
         <is>
@@ -3982,10 +3801,8 @@
           <t>DAVID FERNANDES DA CRUZ</t>
         </is>
       </c>
-      <c r="J47" t="inlineStr">
-        <is>
-          <t>19</t>
-        </is>
+      <c r="J47" t="n">
+        <v>19</v>
       </c>
       <c r="K47" t="n">
         <v>227</v>
@@ -4038,10 +3855,8 @@
           <t>21:28</t>
         </is>
       </c>
-      <c r="F48" t="inlineStr">
-        <is>
-          <t>43463</t>
-        </is>
+      <c r="F48" t="n">
+        <v>43463</v>
       </c>
       <c r="G48" t="inlineStr">
         <is>
@@ -4058,10 +3873,8 @@
           <t>DAVID FERNANDES DA CRUZ</t>
         </is>
       </c>
-      <c r="J48" t="inlineStr">
-        <is>
-          <t>155</t>
-        </is>
+      <c r="J48" t="n">
+        <v>155</v>
       </c>
       <c r="K48" t="n">
         <v>103</v>
@@ -4114,10 +3927,8 @@
           <t>21:34</t>
         </is>
       </c>
-      <c r="F49" t="inlineStr">
-        <is>
-          <t>43470</t>
-        </is>
+      <c r="F49" t="n">
+        <v>43470</v>
       </c>
       <c r="G49" t="inlineStr">
         <is>
@@ -4134,10 +3945,8 @@
           <t>MATEUS AUGUSTO NASCIMENTO COSTA</t>
         </is>
       </c>
-      <c r="J49" t="inlineStr">
-        <is>
-          <t>260</t>
-        </is>
+      <c r="J49" t="n">
+        <v>260</v>
       </c>
       <c r="K49" t="n">
         <v>103</v>
@@ -4190,10 +3999,8 @@
           <t>21:59</t>
         </is>
       </c>
-      <c r="F50" t="inlineStr">
-        <is>
-          <t>43480</t>
-        </is>
+      <c r="F50" t="n">
+        <v>43480</v>
       </c>
       <c r="G50" t="inlineStr">
         <is>
@@ -4210,10 +4017,8 @@
           <t>DAVID FERNANDES DA CRUZ</t>
         </is>
       </c>
-      <c r="J50" t="inlineStr">
-        <is>
-          <t>181</t>
-        </is>
+      <c r="J50" t="n">
+        <v>181</v>
       </c>
       <c r="K50" t="n">
         <v>54</v>
@@ -4266,10 +4071,8 @@
           <t>22:10</t>
         </is>
       </c>
-      <c r="F51" t="inlineStr">
-        <is>
-          <t>43489</t>
-        </is>
+      <c r="F51" t="n">
+        <v>43489</v>
       </c>
       <c r="G51" t="inlineStr">
         <is>
@@ -4286,10 +4089,8 @@
           <t xml:space="preserve">DANIEL BACELAR XAVIER </t>
         </is>
       </c>
-      <c r="J51" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
+      <c r="J51" t="n">
+        <v>4</v>
       </c>
       <c r="K51" t="n">
         <v>170</v>
@@ -4342,10 +4143,8 @@
           <t>22:33</t>
         </is>
       </c>
-      <c r="F52" t="inlineStr">
-        <is>
-          <t>43502</t>
-        </is>
+      <c r="F52" t="n">
+        <v>43502</v>
       </c>
       <c r="G52" t="inlineStr">
         <is>
@@ -4362,10 +4161,8 @@
           <t>DAVID FERNANDES DA CRUZ</t>
         </is>
       </c>
-      <c r="J52" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
+      <c r="J52" t="n">
+        <v>5</v>
       </c>
       <c r="K52" t="n">
         <v>136</v>
@@ -4418,10 +4215,8 @@
           <t>22:33</t>
         </is>
       </c>
-      <c r="F53" t="inlineStr">
-        <is>
-          <t>43501</t>
-        </is>
+      <c r="F53" t="n">
+        <v>43501</v>
       </c>
       <c r="G53" t="inlineStr">
         <is>
@@ -4438,10 +4233,8 @@
           <t>CAIO VINICIUS DOS SANTOS SILVA</t>
         </is>
       </c>
-      <c r="J53" t="inlineStr">
-        <is>
-          <t>28</t>
-        </is>
+      <c r="J53" t="n">
+        <v>28</v>
       </c>
       <c r="K53" t="n">
         <v>170</v>
@@ -4494,10 +4287,8 @@
           <t>22:49</t>
         </is>
       </c>
-      <c r="F54" t="inlineStr">
-        <is>
-          <t>43506</t>
-        </is>
+      <c r="F54" t="n">
+        <v>43506</v>
       </c>
       <c r="G54" t="inlineStr">
         <is>
@@ -4514,10 +4305,8 @@
           <t>DAVID FERNANDES DA CRUZ</t>
         </is>
       </c>
-      <c r="J54" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="J54" t="n">
+        <v>1</v>
       </c>
       <c r="K54" t="n">
         <v>115</v>
@@ -4570,10 +4359,8 @@
           <t>22:49</t>
         </is>
       </c>
-      <c r="F55" t="inlineStr">
-        <is>
-          <t>43507</t>
-        </is>
+      <c r="F55" t="n">
+        <v>43507</v>
       </c>
       <c r="G55" t="inlineStr">
         <is>
@@ -4590,10 +4377,8 @@
           <t>MATEUS AUGUSTO NASCIMENTO COSTA</t>
         </is>
       </c>
-      <c r="J55" t="inlineStr">
-        <is>
-          <t>141</t>
-        </is>
+      <c r="J55" t="n">
+        <v>141</v>
       </c>
       <c r="K55" t="n">
         <v>307</v>
@@ -4646,10 +4431,8 @@
           <t>20:11</t>
         </is>
       </c>
-      <c r="F56" t="inlineStr">
-        <is>
-          <t>43593</t>
-        </is>
+      <c r="F56" t="n">
+        <v>43593</v>
       </c>
       <c r="G56" t="inlineStr">
         <is>
@@ -4666,10 +4449,8 @@
           <t>DAVID FERNANDES DA CRUZ</t>
         </is>
       </c>
-      <c r="J56" t="inlineStr">
-        <is>
-          <t>32</t>
-        </is>
+      <c r="J56" t="n">
+        <v>32</v>
       </c>
       <c r="K56" t="n">
         <v>178.5</v>
@@ -4722,10 +4503,8 @@
           <t>20:36</t>
         </is>
       </c>
-      <c r="F57" t="inlineStr">
-        <is>
-          <t>43596</t>
-        </is>
+      <c r="F57" t="n">
+        <v>43596</v>
       </c>
       <c r="G57" t="inlineStr">
         <is>
@@ -4742,10 +4521,8 @@
           <t>MATEUS AUGUSTO NASCIMENTO COSTA</t>
         </is>
       </c>
-      <c r="J57" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+      <c r="J57" t="n">
+        <v>3</v>
       </c>
       <c r="K57" t="n">
         <v>174</v>
@@ -4798,10 +4575,8 @@
           <t>20:59</t>
         </is>
       </c>
-      <c r="F58" t="inlineStr">
-        <is>
-          <t>43604</t>
-        </is>
+      <c r="F58" t="n">
+        <v>43604</v>
       </c>
       <c r="G58" t="inlineStr">
         <is>
@@ -4818,10 +4593,8 @@
           <t>MATEUS AUGUSTO NASCIMENTO COSTA</t>
         </is>
       </c>
-      <c r="J58" t="inlineStr">
-        <is>
-          <t>12</t>
-        </is>
+      <c r="J58" t="n">
+        <v>12</v>
       </c>
       <c r="K58" t="n">
         <v>133.5</v>
@@ -4874,10 +4647,8 @@
           <t>22:00</t>
         </is>
       </c>
-      <c r="F59" t="inlineStr">
-        <is>
-          <t>43639</t>
-        </is>
+      <c r="F59" t="n">
+        <v>43639</v>
       </c>
       <c r="G59" t="inlineStr">
         <is>
@@ -4894,10 +4665,8 @@
           <t>LUCAS DE MUSSI PALMA</t>
         </is>
       </c>
-      <c r="J59" t="inlineStr">
-        <is>
-          <t>231</t>
-        </is>
+      <c r="J59" t="n">
+        <v>231</v>
       </c>
       <c r="K59" t="n">
         <v>107</v>
@@ -4950,10 +4719,8 @@
           <t>22:03</t>
         </is>
       </c>
-      <c r="F60" t="inlineStr">
-        <is>
-          <t>43643</t>
-        </is>
+      <c r="F60" t="n">
+        <v>43643</v>
       </c>
       <c r="G60" t="inlineStr">
         <is>
@@ -4970,10 +4737,8 @@
           <t>KEROLAINY LAWANY RIO BRANCO</t>
         </is>
       </c>
-      <c r="J60" t="inlineStr">
-        <is>
-          <t>182</t>
-        </is>
+      <c r="J60" t="n">
+        <v>182</v>
       </c>
       <c r="K60" t="n">
         <v>73</v>
@@ -5026,10 +4791,8 @@
           <t>22:17</t>
         </is>
       </c>
-      <c r="F61" t="inlineStr">
-        <is>
-          <t>43655</t>
-        </is>
+      <c r="F61" t="n">
+        <v>43655</v>
       </c>
       <c r="G61" t="inlineStr">
         <is>
@@ -5046,10 +4809,8 @@
           <t>LUCAS DE MUSSI PALMA</t>
         </is>
       </c>
-      <c r="J61" t="inlineStr">
-        <is>
-          <t>44</t>
-        </is>
+      <c r="J61" t="n">
+        <v>44</v>
       </c>
       <c r="K61" t="n">
         <v>203.5</v>
@@ -5102,10 +4863,8 @@
           <t>22:21</t>
         </is>
       </c>
-      <c r="F62" t="inlineStr">
-        <is>
-          <t>43659</t>
-        </is>
+      <c r="F62" t="n">
+        <v>43659</v>
       </c>
       <c r="G62" t="inlineStr">
         <is>
@@ -5122,10 +4881,8 @@
           <t>KEROLAINY LAWANY RIO BRANCO</t>
         </is>
       </c>
-      <c r="J62" t="inlineStr">
-        <is>
-          <t>39</t>
-        </is>
+      <c r="J62" t="n">
+        <v>39</v>
       </c>
       <c r="K62" t="n">
         <v>191</v>
@@ -5178,10 +4935,8 @@
           <t>22:23</t>
         </is>
       </c>
-      <c r="F63" t="inlineStr">
-        <is>
-          <t>43662</t>
-        </is>
+      <c r="F63" t="n">
+        <v>43662</v>
       </c>
       <c r="G63" t="inlineStr">
         <is>
@@ -5198,10 +4953,8 @@
           <t>MATEUS AUGUSTO NASCIMENTO COSTA</t>
         </is>
       </c>
-      <c r="J63" t="inlineStr">
-        <is>
-          <t>179</t>
-        </is>
+      <c r="J63" t="n">
+        <v>179</v>
       </c>
       <c r="K63" t="n">
         <v>173</v>
@@ -5254,10 +5007,8 @@
           <t>22:26</t>
         </is>
       </c>
-      <c r="F64" t="inlineStr">
-        <is>
-          <t>43666</t>
-        </is>
+      <c r="F64" t="n">
+        <v>43666</v>
       </c>
       <c r="G64" t="inlineStr">
         <is>
@@ -5274,10 +5025,8 @@
           <t xml:space="preserve">DAIANA APARECIDA DOS SANTOS SILVA ALVES </t>
         </is>
       </c>
-      <c r="J64" t="inlineStr">
-        <is>
-          <t>12</t>
-        </is>
+      <c r="J64" t="n">
+        <v>12</v>
       </c>
       <c r="K64" t="n">
         <v>177.5</v>
@@ -5330,10 +5079,8 @@
           <t>22:30</t>
         </is>
       </c>
-      <c r="F65" t="inlineStr">
-        <is>
-          <t>43669</t>
-        </is>
+      <c r="F65" t="n">
+        <v>43669</v>
       </c>
       <c r="G65" t="inlineStr">
         <is>
@@ -5350,10 +5097,8 @@
           <t>LUCAS DE MUSSI PALMA</t>
         </is>
       </c>
-      <c r="J65" t="inlineStr">
-        <is>
-          <t>46</t>
-        </is>
+      <c r="J65" t="n">
+        <v>46</v>
       </c>
       <c r="K65" t="n">
         <v>170.5</v>
@@ -5406,10 +5151,8 @@
           <t>22:34</t>
         </is>
       </c>
-      <c r="F66" t="inlineStr">
-        <is>
-          <t>43672</t>
-        </is>
+      <c r="F66" t="n">
+        <v>43672</v>
       </c>
       <c r="G66" t="inlineStr">
         <is>
@@ -5426,10 +5169,8 @@
           <t>LUCAS DE MUSSI PALMA</t>
         </is>
       </c>
-      <c r="J66" t="inlineStr">
-        <is>
-          <t>18</t>
-        </is>
+      <c r="J66" t="n">
+        <v>18</v>
       </c>
       <c r="K66" t="n">
         <v>164</v>
@@ -5482,10 +5223,8 @@
           <t>20:34</t>
         </is>
       </c>
-      <c r="F67" t="inlineStr">
-        <is>
-          <t>43863</t>
-        </is>
+      <c r="F67" t="n">
+        <v>43863</v>
       </c>
       <c r="G67" t="inlineStr">
         <is>
@@ -5502,10 +5241,8 @@
           <t>CAIO VINICIUS DOS SANTOS SILVA</t>
         </is>
       </c>
-      <c r="J67" t="inlineStr">
-        <is>
-          <t>17</t>
-        </is>
+      <c r="J67" t="n">
+        <v>17</v>
       </c>
       <c r="K67" t="n">
         <v>95</v>
@@ -5558,10 +5295,8 @@
           <t>20:36</t>
         </is>
       </c>
-      <c r="F68" t="inlineStr">
-        <is>
-          <t>43865</t>
-        </is>
+      <c r="F68" t="n">
+        <v>43865</v>
       </c>
       <c r="G68" t="inlineStr">
         <is>
@@ -5578,10 +5313,8 @@
           <t>DAVID FERNANDES DA CRUZ</t>
         </is>
       </c>
-      <c r="J68" t="inlineStr">
-        <is>
-          <t>31</t>
-        </is>
+      <c r="J68" t="n">
+        <v>31</v>
       </c>
       <c r="K68" t="n">
         <v>110</v>
@@ -5634,10 +5367,8 @@
           <t>21:58</t>
         </is>
       </c>
-      <c r="F69" t="inlineStr">
-        <is>
-          <t>43898</t>
-        </is>
+      <c r="F69" t="n">
+        <v>43898</v>
       </c>
       <c r="G69" t="inlineStr">
         <is>
@@ -5654,10 +5385,8 @@
           <t>MATEUS AUGUSTO NASCIMENTO COSTA</t>
         </is>
       </c>
-      <c r="J69" t="inlineStr">
-        <is>
-          <t>12</t>
-        </is>
+      <c r="J69" t="n">
+        <v>12</v>
       </c>
       <c r="K69" t="n">
         <v>271</v>
@@ -5710,10 +5439,8 @@
           <t>22:36</t>
         </is>
       </c>
-      <c r="F70" t="inlineStr">
-        <is>
-          <t>43919</t>
-        </is>
+      <c r="F70" t="n">
+        <v>43919</v>
       </c>
       <c r="G70" t="inlineStr">
         <is>
@@ -5730,10 +5457,8 @@
           <t>MATEUS AUGUSTO NASCIMENTO COSTA</t>
         </is>
       </c>
-      <c r="J70" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
+      <c r="J70" t="n">
+        <v>6</v>
       </c>
       <c r="K70" t="n">
         <v>316.5</v>
@@ -5786,10 +5511,8 @@
           <t>23:01</t>
         </is>
       </c>
-      <c r="F71" t="inlineStr">
-        <is>
-          <t>43933</t>
-        </is>
+      <c r="F71" t="n">
+        <v>43933</v>
       </c>
       <c r="G71" t="inlineStr">
         <is>
@@ -5806,10 +5529,8 @@
           <t>DAVID FERNANDES DA CRUZ</t>
         </is>
       </c>
-      <c r="J71" t="inlineStr">
-        <is>
-          <t>14</t>
-        </is>
+      <c r="J71" t="n">
+        <v>14</v>
       </c>
       <c r="K71" t="n">
         <v>349.5</v>
@@ -5862,10 +5583,8 @@
           <t>22:22</t>
         </is>
       </c>
-      <c r="F72" t="inlineStr">
-        <is>
-          <t>43992</t>
-        </is>
+      <c r="F72" t="n">
+        <v>43992</v>
       </c>
       <c r="G72" t="inlineStr">
         <is>
@@ -5930,10 +5649,8 @@
           <t>19:38</t>
         </is>
       </c>
-      <c r="F73" t="inlineStr">
-        <is>
-          <t>44045</t>
-        </is>
+      <c r="F73" t="n">
+        <v>44045</v>
       </c>
       <c r="G73" t="inlineStr">
         <is>
@@ -6002,10 +5719,8 @@
           <t>20:58</t>
         </is>
       </c>
-      <c r="F74" t="inlineStr">
-        <is>
-          <t>44050</t>
-        </is>
+      <c r="F74" t="n">
+        <v>44050</v>
       </c>
       <c r="G74" t="inlineStr">
         <is>
@@ -6074,10 +5789,8 @@
           <t>21:11</t>
         </is>
       </c>
-      <c r="F75" t="inlineStr">
-        <is>
-          <t>44053</t>
-        </is>
+      <c r="F75" t="n">
+        <v>44053</v>
       </c>
       <c r="G75" t="inlineStr">
         <is>
@@ -6146,10 +5859,8 @@
           <t>21:50</t>
         </is>
       </c>
-      <c r="F76" t="inlineStr">
-        <is>
-          <t>44062</t>
-        </is>
+      <c r="F76" t="n">
+        <v>44062</v>
       </c>
       <c r="G76" t="inlineStr">
         <is>
@@ -6218,10 +5929,8 @@
           <t>21:57</t>
         </is>
       </c>
-      <c r="F77" t="inlineStr">
-        <is>
-          <t>44066</t>
-        </is>
+      <c r="F77" t="n">
+        <v>44066</v>
       </c>
       <c r="G77" t="inlineStr">
         <is>
@@ -6290,10 +5999,8 @@
           <t>19:57</t>
         </is>
       </c>
-      <c r="F78" t="inlineStr">
-        <is>
-          <t>44136</t>
-        </is>
+      <c r="F78" t="n">
+        <v>44136</v>
       </c>
       <c r="G78" t="inlineStr">
         <is>
@@ -6362,10 +6069,8 @@
           <t>20:05</t>
         </is>
       </c>
-      <c r="F79" t="inlineStr">
-        <is>
-          <t>44138</t>
-        </is>
+      <c r="F79" t="n">
+        <v>44138</v>
       </c>
       <c r="G79" t="inlineStr">
         <is>
@@ -6434,10 +6139,8 @@
           <t>21:17</t>
         </is>
       </c>
-      <c r="F80" t="inlineStr">
-        <is>
-          <t>44157</t>
-        </is>
+      <c r="F80" t="n">
+        <v>44157</v>
       </c>
       <c r="G80" t="inlineStr">
         <is>
@@ -6506,10 +6209,8 @@
           <t>21:38</t>
         </is>
       </c>
-      <c r="F81" t="inlineStr">
-        <is>
-          <t>44163</t>
-        </is>
+      <c r="F81" t="n">
+        <v>44163</v>
       </c>
       <c r="G81" t="inlineStr">
         <is>
@@ -6578,10 +6279,8 @@
           <t>21:44</t>
         </is>
       </c>
-      <c r="F82" t="inlineStr">
-        <is>
-          <t>44170</t>
-        </is>
+      <c r="F82" t="n">
+        <v>44170</v>
       </c>
       <c r="G82" t="inlineStr">
         <is>
@@ -6650,10 +6349,8 @@
           <t>23:07</t>
         </is>
       </c>
-      <c r="F83" t="inlineStr">
-        <is>
-          <t>44220</t>
-        </is>
+      <c r="F83" t="n">
+        <v>44220</v>
       </c>
       <c r="G83" t="inlineStr">
         <is>
@@ -6696,409 +6393,511 @@
         </is>
       </c>
     </row>
-    <row r="84">
-      <c r="A84" t="inlineStr">
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:P7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="21" customWidth="1" min="7" max="7"/>
+    <col width="27" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="11" customWidth="1" min="11" max="11"/>
+    <col width="15" customWidth="1" min="12" max="12"/>
+    <col width="32" customWidth="1" min="13" max="13"/>
+    <col width="14" customWidth="1" min="14" max="14"/>
+    <col width="10" customWidth="1" min="15" max="15"/>
+    <col width="13" customWidth="1" min="16" max="16"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Loja</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Forma</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Data</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Dia</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Hora PDV</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Cupom</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Caixa</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Operador do caixa</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Atendente</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Mesa</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>Valor PDV</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>Valor máquina</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>Cobrado a mais na máquina (R$)</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>Hora máquina</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>Terminal</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>Autorização</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
         <is>
           <t>ISAIAS 02 - ALPHAVILLE</t>
         </is>
       </c>
-      <c r="B84" t="inlineStr">
+      <c r="B2" t="inlineStr">
         <is>
           <t>Crédito</t>
         </is>
       </c>
-      <c r="C84" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>10/10/2026</t>
         </is>
       </c>
-      <c r="D84" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>sáb</t>
         </is>
       </c>
-      <c r="E84" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>21:26</t>
         </is>
       </c>
-      <c r="F84" t="inlineStr">
-        <is>
-          <t>42146</t>
-        </is>
-      </c>
-      <c r="G84" t="inlineStr">
+      <c r="F2" t="n">
+        <v>42146</v>
+      </c>
+      <c r="G2" t="inlineStr">
         <is>
           <t>001 - IS02 - PDV 01</t>
         </is>
       </c>
-      <c r="H84" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>(analítico não exportado)</t>
         </is>
       </c>
-      <c r="I84" t="inlineStr"/>
-      <c r="J84" t="inlineStr"/>
-      <c r="K84" t="n">
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="n">
         <v>379.5</v>
       </c>
-      <c r="L84" t="n">
+      <c r="L2" t="n">
         <v>417.45</v>
       </c>
-      <c r="M84" t="n">
+      <c r="M2" t="n">
         <v>37.95</v>
       </c>
-      <c r="N84" t="inlineStr">
+      <c r="N2" t="inlineStr">
         <is>
           <t>21:23</t>
         </is>
       </c>
-      <c r="O84" t="inlineStr">
+      <c r="O2" t="inlineStr">
         <is>
           <t>APT88F39</t>
         </is>
       </c>
-      <c r="P84" t="inlineStr">
+      <c r="P2" t="inlineStr">
         <is>
           <t>233482</t>
         </is>
       </c>
     </row>
-    <row r="85">
-      <c r="A85" t="inlineStr">
+    <row r="3">
+      <c r="A3" t="inlineStr">
         <is>
           <t>ISAIAS 02 - ALPHAVILLE</t>
         </is>
       </c>
-      <c r="B85" t="inlineStr">
+      <c r="B3" t="inlineStr">
         <is>
           <t>Crédito</t>
         </is>
       </c>
-      <c r="C85" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
           <t>10/10/2026</t>
         </is>
       </c>
-      <c r="D85" t="inlineStr">
+      <c r="D3" t="inlineStr">
         <is>
           <t>sáb</t>
         </is>
       </c>
-      <c r="E85" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t>22:27</t>
         </is>
       </c>
-      <c r="F85" t="inlineStr">
-        <is>
-          <t>42162</t>
-        </is>
-      </c>
-      <c r="G85" t="inlineStr">
+      <c r="F3" t="n">
+        <v>42162</v>
+      </c>
+      <c r="G3" t="inlineStr">
         <is>
           <t>001 - IS02 - PDV 01</t>
         </is>
       </c>
-      <c r="H85" t="inlineStr">
+      <c r="H3" t="inlineStr">
         <is>
           <t>(analítico não exportado)</t>
         </is>
       </c>
-      <c r="I85" t="inlineStr"/>
-      <c r="J85" t="inlineStr"/>
-      <c r="K85" t="n">
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="n">
         <v>90</v>
       </c>
-      <c r="L85" t="n">
+      <c r="L3" t="n">
         <v>99</v>
       </c>
-      <c r="M85" t="n">
+      <c r="M3" t="n">
         <v>9</v>
       </c>
-      <c r="N85" t="inlineStr">
+      <c r="N3" t="inlineStr">
         <is>
           <t>22:22</t>
         </is>
       </c>
-      <c r="O85" t="inlineStr">
+      <c r="O3" t="inlineStr">
         <is>
           <t>APT88F39</t>
         </is>
       </c>
-      <c r="P85" t="inlineStr">
+      <c r="P3" t="inlineStr">
         <is>
           <t>055764</t>
         </is>
       </c>
     </row>
-    <row r="86">
-      <c r="A86" t="inlineStr">
+    <row r="4">
+      <c r="A4" t="inlineStr">
         <is>
           <t>ISAIAS 02 - ALPHAVILLE</t>
         </is>
       </c>
-      <c r="B86" t="inlineStr">
+      <c r="B4" t="inlineStr">
         <is>
           <t>Débito</t>
         </is>
       </c>
-      <c r="C86" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>15/10/2026</t>
         </is>
       </c>
-      <c r="D86" t="inlineStr">
+      <c r="D4" t="inlineStr">
         <is>
           <t>qui</t>
         </is>
       </c>
-      <c r="E86" t="inlineStr">
+      <c r="E4" t="inlineStr">
         <is>
           <t>19:18</t>
         </is>
       </c>
-      <c r="F86" t="inlineStr">
-        <is>
-          <t>42685</t>
-        </is>
-      </c>
-      <c r="G86" t="inlineStr">
+      <c r="F4" t="n">
+        <v>42685</v>
+      </c>
+      <c r="G4" t="inlineStr">
         <is>
           <t>001 - IS02 - PDV 01</t>
         </is>
       </c>
-      <c r="H86" t="inlineStr">
+      <c r="H4" t="inlineStr">
         <is>
           <t>(analítico não exportado)</t>
         </is>
       </c>
-      <c r="I86" t="inlineStr"/>
-      <c r="J86" t="inlineStr"/>
-      <c r="K86" t="n">
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="n">
         <v>89</v>
       </c>
-      <c r="L86" t="n">
+      <c r="L4" t="n">
         <v>97.90000000000001</v>
       </c>
-      <c r="M86" t="n">
+      <c r="M4" t="n">
         <v>8.9</v>
       </c>
-      <c r="N86" t="inlineStr">
+      <c r="N4" t="inlineStr">
         <is>
           <t>19:17</t>
         </is>
       </c>
-      <c r="O86" t="inlineStr">
+      <c r="O4" t="inlineStr">
         <is>
           <t>APT88F3D</t>
         </is>
       </c>
-      <c r="P86" t="inlineStr">
+      <c r="P4" t="inlineStr">
         <is>
           <t>i0Z97S</t>
         </is>
       </c>
     </row>
-    <row r="87">
-      <c r="A87" t="inlineStr">
+    <row r="5">
+      <c r="A5" t="inlineStr">
         <is>
           <t>ISAIAS 02 - ALPHAVILLE</t>
         </is>
       </c>
-      <c r="B87" t="inlineStr">
+      <c r="B5" t="inlineStr">
         <is>
           <t>Crédito</t>
         </is>
       </c>
-      <c r="C87" t="inlineStr">
+      <c r="C5" t="inlineStr">
         <is>
           <t>15/10/2026</t>
         </is>
       </c>
-      <c r="D87" t="inlineStr">
+      <c r="D5" t="inlineStr">
         <is>
           <t>qui</t>
         </is>
       </c>
-      <c r="E87" t="inlineStr">
+      <c r="E5" t="inlineStr">
         <is>
           <t>21:00</t>
         </is>
       </c>
-      <c r="F87" t="inlineStr">
-        <is>
-          <t>42689</t>
-        </is>
-      </c>
-      <c r="G87" t="inlineStr">
+      <c r="F5" t="n">
+        <v>42689</v>
+      </c>
+      <c r="G5" t="inlineStr">
         <is>
           <t>001 - IS02 - PDV 01</t>
         </is>
       </c>
-      <c r="H87" t="inlineStr">
+      <c r="H5" t="inlineStr">
         <is>
           <t>(analítico não exportado)</t>
         </is>
       </c>
-      <c r="I87" t="inlineStr"/>
-      <c r="J87" t="inlineStr"/>
-      <c r="K87" t="n">
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="n">
         <v>134</v>
       </c>
-      <c r="L87" t="n">
+      <c r="L5" t="n">
         <v>147.4</v>
       </c>
-      <c r="M87" t="n">
+      <c r="M5" t="n">
         <v>13.4</v>
       </c>
-      <c r="N87" t="inlineStr">
+      <c r="N5" t="inlineStr">
         <is>
           <t>20:59</t>
         </is>
       </c>
-      <c r="O87" t="inlineStr">
+      <c r="O5" t="inlineStr">
         <is>
           <t>APT88F39</t>
         </is>
       </c>
-      <c r="P87" t="inlineStr">
+      <c r="P5" t="inlineStr">
         <is>
           <t>883579</t>
         </is>
       </c>
     </row>
-    <row r="88">
-      <c r="A88" t="inlineStr">
+    <row r="6">
+      <c r="A6" t="inlineStr">
         <is>
           <t>ISAIAS 02 - ALPHAVILLE</t>
         </is>
       </c>
-      <c r="B88" t="inlineStr">
+      <c r="B6" t="inlineStr">
         <is>
           <t>Crédito</t>
         </is>
       </c>
-      <c r="C88" t="inlineStr">
+      <c r="C6" t="inlineStr">
         <is>
           <t>18/10/2026</t>
         </is>
       </c>
-      <c r="D88" t="inlineStr">
+      <c r="D6" t="inlineStr">
         <is>
           <t>dom</t>
         </is>
       </c>
-      <c r="E88" t="inlineStr">
+      <c r="E6" t="inlineStr">
         <is>
           <t>21:43</t>
         </is>
       </c>
-      <c r="F88" t="inlineStr">
-        <is>
-          <t>43112</t>
-        </is>
-      </c>
-      <c r="G88" t="inlineStr">
+      <c r="F6" t="n">
+        <v>43112</v>
+      </c>
+      <c r="G6" t="inlineStr">
         <is>
           <t>001 - IS02 - PDV 01</t>
         </is>
       </c>
-      <c r="H88" t="inlineStr">
+      <c r="H6" t="inlineStr">
         <is>
           <t>(analítico não exportado)</t>
         </is>
       </c>
-      <c r="I88" t="inlineStr"/>
-      <c r="J88" t="inlineStr"/>
-      <c r="K88" t="n">
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="n">
         <v>252.4</v>
       </c>
-      <c r="L88" t="n">
+      <c r="L6" t="n">
         <v>277.64</v>
       </c>
-      <c r="M88" t="n">
+      <c r="M6" t="n">
         <v>25.24</v>
       </c>
-      <c r="N88" t="inlineStr">
+      <c r="N6" t="inlineStr">
         <is>
           <t>21:40</t>
         </is>
       </c>
-      <c r="O88" t="inlineStr">
+      <c r="O6" t="inlineStr">
         <is>
           <t>APT88F3A</t>
         </is>
       </c>
-      <c r="P88" t="inlineStr">
+      <c r="P6" t="inlineStr">
         <is>
           <t>819752</t>
         </is>
       </c>
     </row>
-    <row r="89">
-      <c r="A89" t="inlineStr">
+    <row r="7">
+      <c r="A7" t="inlineStr">
         <is>
           <t>ISAIAS 02 - ALPHAVILLE</t>
         </is>
       </c>
-      <c r="B89" t="inlineStr">
+      <c r="B7" t="inlineStr">
         <is>
           <t>Débito</t>
         </is>
       </c>
-      <c r="C89" t="inlineStr">
+      <c r="C7" t="inlineStr">
         <is>
           <t>18/10/2026</t>
         </is>
       </c>
-      <c r="D89" t="inlineStr">
+      <c r="D7" t="inlineStr">
         <is>
           <t>dom</t>
         </is>
       </c>
-      <c r="E89" t="inlineStr">
+      <c r="E7" t="inlineStr">
         <is>
           <t>22:34</t>
         </is>
       </c>
-      <c r="F89" t="inlineStr">
-        <is>
-          <t>43125</t>
-        </is>
-      </c>
-      <c r="G89" t="inlineStr">
+      <c r="F7" t="n">
+        <v>43125</v>
+      </c>
+      <c r="G7" t="inlineStr">
         <is>
           <t>001 - IS02 - PDV 01</t>
         </is>
       </c>
-      <c r="H89" t="inlineStr">
+      <c r="H7" t="inlineStr">
         <is>
           <t>(analítico não exportado)</t>
         </is>
       </c>
-      <c r="I89" t="inlineStr"/>
-      <c r="J89" t="inlineStr"/>
-      <c r="K89" t="n">
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="n">
         <v>286</v>
       </c>
-      <c r="L89" t="n">
+      <c r="L7" t="n">
         <v>314.6</v>
       </c>
-      <c r="M89" t="n">
+      <c r="M7" t="n">
         <v>28.6</v>
       </c>
-      <c r="N89" t="inlineStr">
+      <c r="N7" t="inlineStr">
         <is>
           <t>22:25</t>
         </is>
       </c>
-      <c r="O89" t="inlineStr">
+      <c r="O7" t="inlineStr">
         <is>
           <t>APT88F39</t>
         </is>
       </c>
-      <c r="P89" t="inlineStr">
+      <c r="P7" t="inlineStr">
         <is>
           <t>661429</t>
         </is>

</xml_diff>

<commit_message>
taxa_servico: chave do analítico inclui o caixa (cupom repete entre caixas)
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015XeuzNyreGoe8Jd1wBUgeX
</commit_message>
<xml_diff>
--- a/saida/isaias_taxa_servico_2026-10-01_a_18.xlsx
+++ b/saida/isaias_taxa_servico_2026-10-01_a_18.xlsx
@@ -543,8 +543,10 @@
           <t>18:11</t>
         </is>
       </c>
-      <c r="F2" t="n">
-        <v>42804</v>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>42804</t>
+        </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -561,8 +563,10 @@
           <t>JOSE HENRIQUE ROSA</t>
         </is>
       </c>
-      <c r="J2" t="n">
-        <v>14</v>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
       </c>
       <c r="K2" t="n">
         <v>269</v>
@@ -615,8 +619,10 @@
           <t>20:11</t>
         </is>
       </c>
-      <c r="F3" t="n">
-        <v>42817</v>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>42817</t>
+        </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
@@ -633,8 +639,10 @@
           <t>MATEUS AUGUSTO NASCIMENTO COSTA</t>
         </is>
       </c>
-      <c r="J3" t="n">
-        <v>30</v>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
       </c>
       <c r="K3" t="n">
         <v>160</v>
@@ -687,8 +695,10 @@
           <t>21:06</t>
         </is>
       </c>
-      <c r="F4" t="n">
-        <v>42818</v>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>42818</t>
+        </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
@@ -705,8 +715,10 @@
           <t>MATEUS AUGUSTO NASCIMENTO COSTA</t>
         </is>
       </c>
-      <c r="J4" t="n">
-        <v>29</v>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
       </c>
       <c r="K4" t="n">
         <v>244</v>
@@ -759,8 +771,10 @@
           <t>21:24</t>
         </is>
       </c>
-      <c r="F5" t="n">
-        <v>42823</v>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>42823</t>
+        </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
@@ -777,8 +791,10 @@
           <t>CAIO VINICIUS DOS SANTOS SILVA</t>
         </is>
       </c>
-      <c r="J5" t="n">
-        <v>30</v>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
       </c>
       <c r="K5" t="n">
         <v>88</v>
@@ -831,8 +847,10 @@
           <t>20:33</t>
         </is>
       </c>
-      <c r="F6" t="n">
-        <v>42877</v>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>42877</t>
+        </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
@@ -849,8 +867,10 @@
           <t>KEROLAINY LAWANY RIO BRANCO</t>
         </is>
       </c>
-      <c r="J6" t="n">
-        <v>7</v>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
       </c>
       <c r="K6" t="n">
         <v>151</v>
@@ -903,8 +923,10 @@
           <t>21:15</t>
         </is>
       </c>
-      <c r="F7" t="n">
-        <v>42879</v>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>42879</t>
+        </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
@@ -921,8 +943,10 @@
           <t>LUCAS DE MUSSI PALMA</t>
         </is>
       </c>
-      <c r="J7" t="n">
-        <v>3</v>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="K7" t="n">
         <v>213.5</v>
@@ -975,8 +999,10 @@
           <t>21:31</t>
         </is>
       </c>
-      <c r="F8" t="n">
-        <v>42884</v>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>42884</t>
+        </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
@@ -993,8 +1019,10 @@
           <t>KEROLAINY LAWANY RIO BRANCO</t>
         </is>
       </c>
-      <c r="J8" t="n">
-        <v>30</v>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
       </c>
       <c r="K8" t="n">
         <v>168.5</v>
@@ -1047,8 +1075,10 @@
           <t>21:43</t>
         </is>
       </c>
-      <c r="F9" t="n">
-        <v>42887</v>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>42887</t>
+        </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
@@ -1065,8 +1095,10 @@
           <t>KEROLAINY LAWANY RIO BRANCO</t>
         </is>
       </c>
-      <c r="J9" t="n">
-        <v>26</v>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
       </c>
       <c r="K9" t="n">
         <v>107.5</v>
@@ -1119,8 +1151,10 @@
           <t>21:58</t>
         </is>
       </c>
-      <c r="F10" t="n">
-        <v>42891</v>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>42891</t>
+        </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
@@ -1137,8 +1171,10 @@
           <t>DAVID FERNANDES DA CRUZ</t>
         </is>
       </c>
-      <c r="J10" t="n">
-        <v>5</v>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="K10" t="n">
         <v>150</v>
@@ -1191,8 +1227,10 @@
           <t>21:59</t>
         </is>
       </c>
-      <c r="F11" t="n">
-        <v>42892</v>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>42892</t>
+        </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
@@ -1209,8 +1247,10 @@
           <t>DAVID FERNANDES DA CRUZ</t>
         </is>
       </c>
-      <c r="J11" t="n">
-        <v>7</v>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
       </c>
       <c r="K11" t="n">
         <v>136.5</v>
@@ -1263,8 +1303,10 @@
           <t>22:03</t>
         </is>
       </c>
-      <c r="F12" t="n">
-        <v>42895</v>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>42895</t>
+        </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
@@ -1281,8 +1323,10 @@
           <t xml:space="preserve">DAIANA APARECIDA DOS SANTOS SILVA ALVES </t>
         </is>
       </c>
-      <c r="J12" t="n">
-        <v>252</v>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>252</t>
+        </is>
       </c>
       <c r="K12" t="n">
         <v>277</v>
@@ -1335,8 +1379,10 @@
           <t>22:06</t>
         </is>
       </c>
-      <c r="F13" t="n">
-        <v>42897</v>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>42897</t>
+        </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
@@ -1353,8 +1399,10 @@
           <t>KEROLAINY LAWANY RIO BRANCO</t>
         </is>
       </c>
-      <c r="J13" t="n">
-        <v>152</v>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>152</t>
+        </is>
       </c>
       <c r="K13" t="n">
         <v>104</v>
@@ -1407,8 +1455,10 @@
           <t>22:28</t>
         </is>
       </c>
-      <c r="F14" t="n">
-        <v>42902</v>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>42902</t>
+        </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
@@ -1425,8 +1475,10 @@
           <t xml:space="preserve">DAIANA APARECIDA DOS SANTOS SILVA ALVES </t>
         </is>
       </c>
-      <c r="J14" t="n">
-        <v>29</v>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
       </c>
       <c r="K14" t="n">
         <v>213</v>
@@ -1479,8 +1531,10 @@
           <t>22:40</t>
         </is>
       </c>
-      <c r="F15" t="n">
-        <v>42908</v>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>42908</t>
+        </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
@@ -1497,8 +1551,10 @@
           <t xml:space="preserve">DAIANA APARECIDA DOS SANTOS SILVA ALVES </t>
         </is>
       </c>
-      <c r="J15" t="n">
-        <v>244</v>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>244</t>
+        </is>
       </c>
       <c r="K15" t="n">
         <v>517</v>
@@ -1551,8 +1607,10 @@
           <t>23:24</t>
         </is>
       </c>
-      <c r="F16" t="n">
-        <v>42921</v>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>42921</t>
+        </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
@@ -1569,8 +1627,10 @@
           <t xml:space="preserve">DANIEL BACELAR XAVIER </t>
         </is>
       </c>
-      <c r="J16" t="n">
-        <v>18</v>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
       </c>
       <c r="K16" t="n">
         <v>149.5</v>
@@ -1623,8 +1683,10 @@
           <t>21:20</t>
         </is>
       </c>
-      <c r="F17" t="n">
-        <v>42983</v>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>42983</t>
+        </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
@@ -1641,8 +1703,10 @@
           <t xml:space="preserve">DANIEL BACELAR XAVIER </t>
         </is>
       </c>
-      <c r="J17" t="n">
-        <v>266</v>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>266</t>
+        </is>
       </c>
       <c r="K17" t="n">
         <v>135.5</v>
@@ -1695,8 +1759,10 @@
           <t>22:16</t>
         </is>
       </c>
-      <c r="F18" t="n">
-        <v>43013</v>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>43013</t>
+        </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
@@ -1713,8 +1779,10 @@
           <t>CAIO VINICIUS DOS SANTOS SILVA</t>
         </is>
       </c>
-      <c r="J18" t="n">
-        <v>28</v>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
       </c>
       <c r="K18" t="n">
         <v>87</v>
@@ -1767,8 +1835,10 @@
           <t>23:25</t>
         </is>
       </c>
-      <c r="F19" t="n">
-        <v>43068</v>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>43068</t>
+        </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
@@ -1785,8 +1855,10 @@
           <t xml:space="preserve">DANIEL BACELAR XAVIER </t>
         </is>
       </c>
-      <c r="J19" t="n">
-        <v>208</v>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>208</t>
+        </is>
       </c>
       <c r="K19" t="n">
         <v>49</v>
@@ -1839,8 +1911,10 @@
           <t>23:26</t>
         </is>
       </c>
-      <c r="F20" t="n">
-        <v>43070</v>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>43070</t>
+        </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
@@ -1857,8 +1931,10 @@
           <t xml:space="preserve">DANIEL BACELAR XAVIER </t>
         </is>
       </c>
-      <c r="J20" t="n">
-        <v>185</v>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>185</t>
+        </is>
       </c>
       <c r="K20" t="n">
         <v>61</v>
@@ -1911,8 +1987,10 @@
           <t>23:30</t>
         </is>
       </c>
-      <c r="F21" t="n">
-        <v>43076</v>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>43076</t>
+        </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
@@ -1929,8 +2007,10 @@
           <t>MATEUS AUGUSTO NASCIMENTO COSTA</t>
         </is>
       </c>
-      <c r="J21" t="n">
-        <v>6</v>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
       </c>
       <c r="K21" t="n">
         <v>226</v>
@@ -1983,8 +2063,10 @@
           <t>23:30</t>
         </is>
       </c>
-      <c r="F22" t="n">
-        <v>43075</v>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>43075</t>
+        </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
@@ -2001,8 +2083,10 @@
           <t>MATEUS AUGUSTO NASCIMENTO COSTA</t>
         </is>
       </c>
-      <c r="J22" t="n">
-        <v>12</v>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
       </c>
       <c r="K22" t="n">
         <v>148</v>
@@ -2055,8 +2139,10 @@
           <t>23:31</t>
         </is>
       </c>
-      <c r="F23" t="n">
-        <v>43078</v>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>43078</t>
+        </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
@@ -2073,8 +2159,10 @@
           <t>MATEUS AUGUSTO NASCIMENTO COSTA</t>
         </is>
       </c>
-      <c r="J23" t="n">
-        <v>17</v>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
       </c>
       <c r="K23" t="n">
         <v>147.5</v>
@@ -2127,8 +2215,10 @@
           <t>23:45</t>
         </is>
       </c>
-      <c r="F24" t="n">
-        <v>43085</v>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>43085</t>
+        </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
@@ -2145,8 +2235,10 @@
           <t>DAVID FERNANDES DA CRUZ</t>
         </is>
       </c>
-      <c r="J24" t="n">
-        <v>3</v>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="K24" t="n">
         <v>196.5</v>
@@ -2199,8 +2291,10 @@
           <t>20:28</t>
         </is>
       </c>
-      <c r="F25" t="n">
-        <v>43117</v>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>43117</t>
+        </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
@@ -2217,8 +2311,10 @@
           <t>MATEUS AUGUSTO NASCIMENTO COSTA</t>
         </is>
       </c>
-      <c r="J25" t="n">
-        <v>7</v>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
       </c>
       <c r="K25" t="n">
         <v>124</v>
@@ -2271,8 +2367,10 @@
           <t>22:07</t>
         </is>
       </c>
-      <c r="F26" t="n">
-        <v>43138</v>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>43138</t>
+        </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
@@ -2289,8 +2387,10 @@
           <t>KEROLAINY LAWANY RIO BRANCO</t>
         </is>
       </c>
-      <c r="J26" t="n">
-        <v>6</v>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
       </c>
       <c r="K26" t="n">
         <v>94</v>
@@ -2343,8 +2443,10 @@
           <t>22:30</t>
         </is>
       </c>
-      <c r="F27" t="n">
-        <v>43151</v>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>43151</t>
+        </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
@@ -2361,8 +2463,10 @@
           <t>DAVID FERNANDES DA CRUZ</t>
         </is>
       </c>
-      <c r="J27" t="n">
-        <v>31</v>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>31</t>
+        </is>
       </c>
       <c r="K27" t="n">
         <v>105</v>
@@ -2415,8 +2519,10 @@
           <t>22:31</t>
         </is>
       </c>
-      <c r="F28" t="n">
-        <v>43153</v>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>43153</t>
+        </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
@@ -2433,8 +2539,10 @@
           <t>CAIO VINICIUS DOS SANTOS SILVA</t>
         </is>
       </c>
-      <c r="J28" t="n">
-        <v>179</v>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>179</t>
+        </is>
       </c>
       <c r="K28" t="n">
         <v>144</v>
@@ -2487,8 +2595,10 @@
           <t>12:55</t>
         </is>
       </c>
-      <c r="F29" t="n">
-        <v>43179</v>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>43179</t>
+        </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
@@ -2505,8 +2615,10 @@
           <t>CAIO VINICIUS DOS SANTOS SILVA</t>
         </is>
       </c>
-      <c r="J29" t="n">
-        <v>11</v>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
       </c>
       <c r="K29" t="n">
         <v>84</v>
@@ -2559,8 +2671,10 @@
           <t>18:52</t>
         </is>
       </c>
-      <c r="F30" t="n">
-        <v>43212</v>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>43212</t>
+        </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
@@ -2577,8 +2691,10 @@
           <t>JOSE HENRIQUE ROSA</t>
         </is>
       </c>
-      <c r="J30" t="n">
-        <v>15</v>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
       </c>
       <c r="K30" t="n">
         <v>113</v>
@@ -2631,8 +2747,10 @@
           <t>21:16</t>
         </is>
       </c>
-      <c r="F31" t="n">
-        <v>43219</v>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>43219</t>
+        </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
@@ -2649,8 +2767,10 @@
           <t xml:space="preserve">DAIANA APARECIDA DOS SANTOS SILVA ALVES </t>
         </is>
       </c>
-      <c r="J31" t="n">
-        <v>29</v>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
       </c>
       <c r="K31" t="n">
         <v>127</v>
@@ -2703,8 +2823,10 @@
           <t>21:24</t>
         </is>
       </c>
-      <c r="F32" t="n">
-        <v>43222</v>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>43222</t>
+        </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
@@ -2721,8 +2843,10 @@
           <t xml:space="preserve">DAIANA APARECIDA DOS SANTOS SILVA ALVES </t>
         </is>
       </c>
-      <c r="J32" t="n">
-        <v>157</v>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>157</t>
+        </is>
       </c>
       <c r="K32" t="n">
         <v>50</v>
@@ -2775,8 +2899,10 @@
           <t>22:26</t>
         </is>
       </c>
-      <c r="F33" t="n">
-        <v>43316</v>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>43316</t>
+        </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
@@ -2793,8 +2919,10 @@
           <t xml:space="preserve">DANIEL BACELAR XAVIER </t>
         </is>
       </c>
-      <c r="J33" t="n">
-        <v>6</v>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
       </c>
       <c r="K33" t="n">
         <v>143.5</v>
@@ -2847,8 +2975,10 @@
           <t>22:56</t>
         </is>
       </c>
-      <c r="F34" t="n">
-        <v>43322</v>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>43322</t>
+        </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
@@ -2865,8 +2995,10 @@
           <t>DAVID FERNANDES DA CRUZ</t>
         </is>
       </c>
-      <c r="J34" t="n">
-        <v>30</v>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
       </c>
       <c r="K34" t="n">
         <v>93</v>
@@ -2919,8 +3051,10 @@
           <t>20:42</t>
         </is>
       </c>
-      <c r="F35" t="n">
-        <v>43366</v>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>43366</t>
+        </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
@@ -2937,8 +3071,10 @@
           <t>MATEUS AUGUSTO NASCIMENTO COSTA</t>
         </is>
       </c>
-      <c r="J35" t="n">
-        <v>29</v>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
       </c>
       <c r="K35" t="n">
         <v>110.5</v>
@@ -2991,8 +3127,10 @@
           <t>21:17</t>
         </is>
       </c>
-      <c r="F36" t="n">
-        <v>43370</v>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>43370</t>
+        </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
@@ -3009,8 +3147,10 @@
           <t xml:space="preserve">DAIANA APARECIDA DOS SANTOS SILVA ALVES </t>
         </is>
       </c>
-      <c r="J36" t="n">
-        <v>14</v>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
       </c>
       <c r="K36" t="n">
         <v>124.5</v>
@@ -3063,8 +3203,10 @@
           <t>21:24</t>
         </is>
       </c>
-      <c r="F37" t="n">
-        <v>43372</v>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>43372</t>
+        </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
@@ -3081,8 +3223,10 @@
           <t xml:space="preserve">DAIANA APARECIDA DOS SANTOS SILVA ALVES </t>
         </is>
       </c>
-      <c r="J37" t="n">
-        <v>7</v>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
       </c>
       <c r="K37" t="n">
         <v>159</v>
@@ -3135,8 +3279,10 @@
           <t>21:45</t>
         </is>
       </c>
-      <c r="F38" t="n">
-        <v>43379</v>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>43379</t>
+        </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
@@ -3153,8 +3299,10 @@
           <t xml:space="preserve">DAIANA APARECIDA DOS SANTOS SILVA ALVES </t>
         </is>
       </c>
-      <c r="J38" t="n">
-        <v>28</v>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
       </c>
       <c r="K38" t="n">
         <v>191.5</v>
@@ -3207,8 +3355,10 @@
           <t>21:53</t>
         </is>
       </c>
-      <c r="F39" t="n">
-        <v>43382</v>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>43382</t>
+        </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
@@ -3225,8 +3375,10 @@
           <t>KEROLAINY LAWANY RIO BRANCO</t>
         </is>
       </c>
-      <c r="J39" t="n">
-        <v>31</v>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>31</t>
+        </is>
       </c>
       <c r="K39" t="n">
         <v>153</v>
@@ -3279,8 +3431,10 @@
           <t>23:09</t>
         </is>
       </c>
-      <c r="F40" t="n">
-        <v>43416</v>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>43416</t>
+        </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
@@ -3297,8 +3451,10 @@
           <t>KEROLAINY LAWANY RIO BRANCO</t>
         </is>
       </c>
-      <c r="J40" t="n">
-        <v>7</v>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
       </c>
       <c r="K40" t="n">
         <v>208</v>
@@ -3351,8 +3507,10 @@
           <t>20:11</t>
         </is>
       </c>
-      <c r="F41" t="n">
-        <v>43440</v>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>43440</t>
+        </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
@@ -3369,8 +3527,10 @@
           <t xml:space="preserve">DANIEL BACELAR XAVIER </t>
         </is>
       </c>
-      <c r="J41" t="n">
-        <v>11</v>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
       </c>
       <c r="K41" t="n">
         <v>215</v>
@@ -3423,8 +3583,10 @@
           <t>20:42</t>
         </is>
       </c>
-      <c r="F42" t="n">
-        <v>43444</v>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>43444</t>
+        </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
@@ -3441,8 +3603,10 @@
           <t xml:space="preserve">DANIEL BACELAR XAVIER </t>
         </is>
       </c>
-      <c r="J42" t="n">
-        <v>6</v>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
       </c>
       <c r="K42" t="n">
         <v>226</v>
@@ -3495,8 +3659,10 @@
           <t>21:15</t>
         </is>
       </c>
-      <c r="F43" t="n">
-        <v>43452</v>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>43452</t>
+        </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
@@ -3513,8 +3679,10 @@
           <t>LUCAS DE MUSSI PALMA</t>
         </is>
       </c>
-      <c r="J43" t="n">
-        <v>240</v>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>240</t>
+        </is>
       </c>
       <c r="K43" t="n">
         <v>257</v>
@@ -3567,8 +3735,10 @@
           <t>21:16</t>
         </is>
       </c>
-      <c r="F44" t="n">
-        <v>43454</v>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>43454</t>
+        </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
@@ -3585,8 +3755,10 @@
           <t xml:space="preserve">DANIEL BACELAR XAVIER </t>
         </is>
       </c>
-      <c r="J44" t="n">
-        <v>124</v>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>124</t>
+        </is>
       </c>
       <c r="K44" t="n">
         <v>52</v>
@@ -3639,8 +3811,10 @@
           <t>21:18</t>
         </is>
       </c>
-      <c r="F45" t="n">
-        <v>43456</v>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>43456</t>
+        </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
@@ -3657,8 +3831,10 @@
           <t xml:space="preserve">DANIEL BACELAR XAVIER </t>
         </is>
       </c>
-      <c r="J45" t="n">
-        <v>206</v>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>206</t>
+        </is>
       </c>
       <c r="K45" t="n">
         <v>256</v>
@@ -3711,8 +3887,10 @@
           <t>21:18</t>
         </is>
       </c>
-      <c r="F46" t="n">
-        <v>43457</v>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>43457</t>
+        </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
@@ -3729,8 +3907,10 @@
           <t xml:space="preserve">DANIEL BACELAR XAVIER </t>
         </is>
       </c>
-      <c r="J46" t="n">
-        <v>7</v>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
       </c>
       <c r="K46" t="n">
         <v>282</v>
@@ -3783,8 +3963,10 @@
           <t>21:18</t>
         </is>
       </c>
-      <c r="F47" t="n">
-        <v>43458</v>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>43458</t>
+        </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
@@ -3801,8 +3983,10 @@
           <t>DAVID FERNANDES DA CRUZ</t>
         </is>
       </c>
-      <c r="J47" t="n">
-        <v>19</v>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
       </c>
       <c r="K47" t="n">
         <v>227</v>
@@ -3855,8 +4039,10 @@
           <t>21:28</t>
         </is>
       </c>
-      <c r="F48" t="n">
-        <v>43463</v>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>43463</t>
+        </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
@@ -3873,8 +4059,10 @@
           <t>DAVID FERNANDES DA CRUZ</t>
         </is>
       </c>
-      <c r="J48" t="n">
-        <v>155</v>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>155</t>
+        </is>
       </c>
       <c r="K48" t="n">
         <v>103</v>
@@ -3927,8 +4115,10 @@
           <t>21:34</t>
         </is>
       </c>
-      <c r="F49" t="n">
-        <v>43470</v>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>43470</t>
+        </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
@@ -3945,8 +4135,10 @@
           <t>MATEUS AUGUSTO NASCIMENTO COSTA</t>
         </is>
       </c>
-      <c r="J49" t="n">
-        <v>260</v>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>260</t>
+        </is>
       </c>
       <c r="K49" t="n">
         <v>103</v>
@@ -3999,8 +4191,10 @@
           <t>21:59</t>
         </is>
       </c>
-      <c r="F50" t="n">
-        <v>43480</v>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>43480</t>
+        </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
@@ -4017,8 +4211,10 @@
           <t>DAVID FERNANDES DA CRUZ</t>
         </is>
       </c>
-      <c r="J50" t="n">
-        <v>181</v>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>181</t>
+        </is>
       </c>
       <c r="K50" t="n">
         <v>54</v>
@@ -4071,8 +4267,10 @@
           <t>22:10</t>
         </is>
       </c>
-      <c r="F51" t="n">
-        <v>43489</v>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>43489</t>
+        </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
@@ -4089,8 +4287,10 @@
           <t xml:space="preserve">DANIEL BACELAR XAVIER </t>
         </is>
       </c>
-      <c r="J51" t="n">
-        <v>4</v>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="K51" t="n">
         <v>170</v>
@@ -4143,8 +4343,10 @@
           <t>22:33</t>
         </is>
       </c>
-      <c r="F52" t="n">
-        <v>43502</v>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>43502</t>
+        </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
@@ -4161,8 +4363,10 @@
           <t>DAVID FERNANDES DA CRUZ</t>
         </is>
       </c>
-      <c r="J52" t="n">
-        <v>5</v>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="K52" t="n">
         <v>136</v>
@@ -4215,8 +4419,10 @@
           <t>22:33</t>
         </is>
       </c>
-      <c r="F53" t="n">
-        <v>43501</v>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>43501</t>
+        </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
@@ -4233,8 +4439,10 @@
           <t>CAIO VINICIUS DOS SANTOS SILVA</t>
         </is>
       </c>
-      <c r="J53" t="n">
-        <v>28</v>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
       </c>
       <c r="K53" t="n">
         <v>170</v>
@@ -4287,8 +4495,10 @@
           <t>22:49</t>
         </is>
       </c>
-      <c r="F54" t="n">
-        <v>43506</v>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>43506</t>
+        </is>
       </c>
       <c r="G54" t="inlineStr">
         <is>
@@ -4305,8 +4515,10 @@
           <t>DAVID FERNANDES DA CRUZ</t>
         </is>
       </c>
-      <c r="J54" t="n">
-        <v>1</v>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="K54" t="n">
         <v>115</v>
@@ -4359,8 +4571,10 @@
           <t>22:49</t>
         </is>
       </c>
-      <c r="F55" t="n">
-        <v>43507</v>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>43507</t>
+        </is>
       </c>
       <c r="G55" t="inlineStr">
         <is>
@@ -4377,8 +4591,10 @@
           <t>MATEUS AUGUSTO NASCIMENTO COSTA</t>
         </is>
       </c>
-      <c r="J55" t="n">
-        <v>141</v>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>141</t>
+        </is>
       </c>
       <c r="K55" t="n">
         <v>307</v>
@@ -4431,8 +4647,10 @@
           <t>20:11</t>
         </is>
       </c>
-      <c r="F56" t="n">
-        <v>43593</v>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>43593</t>
+        </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
@@ -4449,8 +4667,10 @@
           <t>DAVID FERNANDES DA CRUZ</t>
         </is>
       </c>
-      <c r="J56" t="n">
-        <v>32</v>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>32</t>
+        </is>
       </c>
       <c r="K56" t="n">
         <v>178.5</v>
@@ -4503,8 +4723,10 @@
           <t>20:36</t>
         </is>
       </c>
-      <c r="F57" t="n">
-        <v>43596</v>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>43596</t>
+        </is>
       </c>
       <c r="G57" t="inlineStr">
         <is>
@@ -4521,8 +4743,10 @@
           <t>MATEUS AUGUSTO NASCIMENTO COSTA</t>
         </is>
       </c>
-      <c r="J57" t="n">
-        <v>3</v>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="K57" t="n">
         <v>174</v>
@@ -4575,8 +4799,10 @@
           <t>20:59</t>
         </is>
       </c>
-      <c r="F58" t="n">
-        <v>43604</v>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>43604</t>
+        </is>
       </c>
       <c r="G58" t="inlineStr">
         <is>
@@ -4593,8 +4819,10 @@
           <t>MATEUS AUGUSTO NASCIMENTO COSTA</t>
         </is>
       </c>
-      <c r="J58" t="n">
-        <v>12</v>
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
       </c>
       <c r="K58" t="n">
         <v>133.5</v>
@@ -4647,8 +4875,10 @@
           <t>22:00</t>
         </is>
       </c>
-      <c r="F59" t="n">
-        <v>43639</v>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>43639</t>
+        </is>
       </c>
       <c r="G59" t="inlineStr">
         <is>
@@ -4665,8 +4895,10 @@
           <t>LUCAS DE MUSSI PALMA</t>
         </is>
       </c>
-      <c r="J59" t="n">
-        <v>231</v>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>231</t>
+        </is>
       </c>
       <c r="K59" t="n">
         <v>107</v>
@@ -4719,8 +4951,10 @@
           <t>22:03</t>
         </is>
       </c>
-      <c r="F60" t="n">
-        <v>43643</v>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>43643</t>
+        </is>
       </c>
       <c r="G60" t="inlineStr">
         <is>
@@ -4737,8 +4971,10 @@
           <t>KEROLAINY LAWANY RIO BRANCO</t>
         </is>
       </c>
-      <c r="J60" t="n">
-        <v>182</v>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>182</t>
+        </is>
       </c>
       <c r="K60" t="n">
         <v>73</v>
@@ -4791,8 +5027,10 @@
           <t>22:17</t>
         </is>
       </c>
-      <c r="F61" t="n">
-        <v>43655</v>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>43655</t>
+        </is>
       </c>
       <c r="G61" t="inlineStr">
         <is>
@@ -4809,8 +5047,10 @@
           <t>LUCAS DE MUSSI PALMA</t>
         </is>
       </c>
-      <c r="J61" t="n">
-        <v>44</v>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>44</t>
+        </is>
       </c>
       <c r="K61" t="n">
         <v>203.5</v>
@@ -4863,8 +5103,10 @@
           <t>22:21</t>
         </is>
       </c>
-      <c r="F62" t="n">
-        <v>43659</v>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>43659</t>
+        </is>
       </c>
       <c r="G62" t="inlineStr">
         <is>
@@ -4881,8 +5123,10 @@
           <t>KEROLAINY LAWANY RIO BRANCO</t>
         </is>
       </c>
-      <c r="J62" t="n">
-        <v>39</v>
+      <c r="J62" t="inlineStr">
+        <is>
+          <t>39</t>
+        </is>
       </c>
       <c r="K62" t="n">
         <v>191</v>
@@ -4935,8 +5179,10 @@
           <t>22:23</t>
         </is>
       </c>
-      <c r="F63" t="n">
-        <v>43662</v>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>43662</t>
+        </is>
       </c>
       <c r="G63" t="inlineStr">
         <is>
@@ -4953,8 +5199,10 @@
           <t>MATEUS AUGUSTO NASCIMENTO COSTA</t>
         </is>
       </c>
-      <c r="J63" t="n">
-        <v>179</v>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>179</t>
+        </is>
       </c>
       <c r="K63" t="n">
         <v>173</v>
@@ -5007,8 +5255,10 @@
           <t>22:26</t>
         </is>
       </c>
-      <c r="F64" t="n">
-        <v>43666</v>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>43666</t>
+        </is>
       </c>
       <c r="G64" t="inlineStr">
         <is>
@@ -5025,8 +5275,10 @@
           <t xml:space="preserve">DAIANA APARECIDA DOS SANTOS SILVA ALVES </t>
         </is>
       </c>
-      <c r="J64" t="n">
-        <v>12</v>
+      <c r="J64" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
       </c>
       <c r="K64" t="n">
         <v>177.5</v>
@@ -5079,8 +5331,10 @@
           <t>22:30</t>
         </is>
       </c>
-      <c r="F65" t="n">
-        <v>43669</v>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>43669</t>
+        </is>
       </c>
       <c r="G65" t="inlineStr">
         <is>
@@ -5097,8 +5351,10 @@
           <t>LUCAS DE MUSSI PALMA</t>
         </is>
       </c>
-      <c r="J65" t="n">
-        <v>46</v>
+      <c r="J65" t="inlineStr">
+        <is>
+          <t>46</t>
+        </is>
       </c>
       <c r="K65" t="n">
         <v>170.5</v>
@@ -5151,8 +5407,10 @@
           <t>22:34</t>
         </is>
       </c>
-      <c r="F66" t="n">
-        <v>43672</v>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>43672</t>
+        </is>
       </c>
       <c r="G66" t="inlineStr">
         <is>
@@ -5169,8 +5427,10 @@
           <t>LUCAS DE MUSSI PALMA</t>
         </is>
       </c>
-      <c r="J66" t="n">
-        <v>18</v>
+      <c r="J66" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
       </c>
       <c r="K66" t="n">
         <v>164</v>
@@ -5223,8 +5483,10 @@
           <t>20:34</t>
         </is>
       </c>
-      <c r="F67" t="n">
-        <v>43863</v>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>43863</t>
+        </is>
       </c>
       <c r="G67" t="inlineStr">
         <is>
@@ -5241,8 +5503,10 @@
           <t>CAIO VINICIUS DOS SANTOS SILVA</t>
         </is>
       </c>
-      <c r="J67" t="n">
-        <v>17</v>
+      <c r="J67" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
       </c>
       <c r="K67" t="n">
         <v>95</v>
@@ -5295,8 +5559,10 @@
           <t>20:36</t>
         </is>
       </c>
-      <c r="F68" t="n">
-        <v>43865</v>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>43865</t>
+        </is>
       </c>
       <c r="G68" t="inlineStr">
         <is>
@@ -5313,8 +5579,10 @@
           <t>DAVID FERNANDES DA CRUZ</t>
         </is>
       </c>
-      <c r="J68" t="n">
-        <v>31</v>
+      <c r="J68" t="inlineStr">
+        <is>
+          <t>31</t>
+        </is>
       </c>
       <c r="K68" t="n">
         <v>110</v>
@@ -5367,8 +5635,10 @@
           <t>21:58</t>
         </is>
       </c>
-      <c r="F69" t="n">
-        <v>43898</v>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>43898</t>
+        </is>
       </c>
       <c r="G69" t="inlineStr">
         <is>
@@ -5385,8 +5655,10 @@
           <t>MATEUS AUGUSTO NASCIMENTO COSTA</t>
         </is>
       </c>
-      <c r="J69" t="n">
-        <v>12</v>
+      <c r="J69" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
       </c>
       <c r="K69" t="n">
         <v>271</v>
@@ -5439,8 +5711,10 @@
           <t>22:36</t>
         </is>
       </c>
-      <c r="F70" t="n">
-        <v>43919</v>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>43919</t>
+        </is>
       </c>
       <c r="G70" t="inlineStr">
         <is>
@@ -5457,8 +5731,10 @@
           <t>MATEUS AUGUSTO NASCIMENTO COSTA</t>
         </is>
       </c>
-      <c r="J70" t="n">
-        <v>6</v>
+      <c r="J70" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
       </c>
       <c r="K70" t="n">
         <v>316.5</v>
@@ -5511,8 +5787,10 @@
           <t>23:01</t>
         </is>
       </c>
-      <c r="F71" t="n">
-        <v>43933</v>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>43933</t>
+        </is>
       </c>
       <c r="G71" t="inlineStr">
         <is>
@@ -5529,8 +5807,10 @@
           <t>DAVID FERNANDES DA CRUZ</t>
         </is>
       </c>
-      <c r="J71" t="n">
-        <v>14</v>
+      <c r="J71" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
       </c>
       <c r="K71" t="n">
         <v>349.5</v>
@@ -5583,8 +5863,10 @@
           <t>22:22</t>
         </is>
       </c>
-      <c r="F72" t="n">
-        <v>43992</v>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>43992</t>
+        </is>
       </c>
       <c r="G72" t="inlineStr">
         <is>
@@ -5649,8 +5931,10 @@
           <t>19:38</t>
         </is>
       </c>
-      <c r="F73" t="n">
-        <v>44045</v>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>44045</t>
+        </is>
       </c>
       <c r="G73" t="inlineStr">
         <is>
@@ -5659,14 +5943,10 @@
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>MARIANA CHAVES</t>
-        </is>
-      </c>
-      <c r="I73" t="inlineStr">
-        <is>
-          <t>ADM ISAIAS 01</t>
-        </is>
-      </c>
+          <t>(analítico não exportado)</t>
+        </is>
+      </c>
+      <c r="I73" t="inlineStr"/>
       <c r="J73" t="inlineStr"/>
       <c r="K73" t="n">
         <v>166.5</v>
@@ -5719,8 +5999,10 @@
           <t>20:58</t>
         </is>
       </c>
-      <c r="F74" t="n">
-        <v>44050</v>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>44050</t>
+        </is>
       </c>
       <c r="G74" t="inlineStr">
         <is>
@@ -5729,14 +6011,10 @@
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>MARIANA CHAVES</t>
-        </is>
-      </c>
-      <c r="I74" t="inlineStr">
-        <is>
-          <t>ADM ISAIAS 01</t>
-        </is>
-      </c>
+          <t>(analítico não exportado)</t>
+        </is>
+      </c>
+      <c r="I74" t="inlineStr"/>
       <c r="J74" t="inlineStr"/>
       <c r="K74" t="n">
         <v>342</v>
@@ -5789,8 +6067,10 @@
           <t>21:11</t>
         </is>
       </c>
-      <c r="F75" t="n">
-        <v>44053</v>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>44053</t>
+        </is>
       </c>
       <c r="G75" t="inlineStr">
         <is>
@@ -5799,14 +6079,10 @@
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>MARIANA CHAVES</t>
-        </is>
-      </c>
-      <c r="I75" t="inlineStr">
-        <is>
-          <t>ADM ISAIAS 01</t>
-        </is>
-      </c>
+          <t>(analítico não exportado)</t>
+        </is>
+      </c>
+      <c r="I75" t="inlineStr"/>
       <c r="J75" t="inlineStr"/>
       <c r="K75" t="n">
         <v>256</v>
@@ -5859,8 +6135,10 @@
           <t>21:50</t>
         </is>
       </c>
-      <c r="F76" t="n">
-        <v>44062</v>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>44062</t>
+        </is>
       </c>
       <c r="G76" t="inlineStr">
         <is>
@@ -5869,14 +6147,10 @@
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>MARIANA CHAVES</t>
-        </is>
-      </c>
-      <c r="I76" t="inlineStr">
-        <is>
-          <t>ADM ISAIAS 01</t>
-        </is>
-      </c>
+          <t>(analítico não exportado)</t>
+        </is>
+      </c>
+      <c r="I76" t="inlineStr"/>
       <c r="J76" t="inlineStr"/>
       <c r="K76" t="n">
         <v>103</v>
@@ -5929,8 +6203,10 @@
           <t>21:57</t>
         </is>
       </c>
-      <c r="F77" t="n">
-        <v>44066</v>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>44066</t>
+        </is>
       </c>
       <c r="G77" t="inlineStr">
         <is>
@@ -5939,14 +6215,10 @@
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>MARIANA CHAVES</t>
-        </is>
-      </c>
-      <c r="I77" t="inlineStr">
-        <is>
-          <t>ADM ISAIAS 01</t>
-        </is>
-      </c>
+          <t>(analítico não exportado)</t>
+        </is>
+      </c>
+      <c r="I77" t="inlineStr"/>
       <c r="J77" t="inlineStr"/>
       <c r="K77" t="n">
         <v>272</v>
@@ -5999,8 +6271,10 @@
           <t>19:57</t>
         </is>
       </c>
-      <c r="F78" t="n">
-        <v>44136</v>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>44136</t>
+        </is>
       </c>
       <c r="G78" t="inlineStr">
         <is>
@@ -6009,14 +6283,10 @@
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>MARIANA CHAVES</t>
-        </is>
-      </c>
-      <c r="I78" t="inlineStr">
-        <is>
-          <t>ADM ISAIAS 01</t>
-        </is>
-      </c>
+          <t>(analítico não exportado)</t>
+        </is>
+      </c>
+      <c r="I78" t="inlineStr"/>
       <c r="J78" t="inlineStr"/>
       <c r="K78" t="n">
         <v>168</v>
@@ -6069,8 +6339,10 @@
           <t>20:05</t>
         </is>
       </c>
-      <c r="F79" t="n">
-        <v>44138</v>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>44138</t>
+        </is>
       </c>
       <c r="G79" t="inlineStr">
         <is>
@@ -6079,14 +6351,10 @@
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>MARIANA CHAVES</t>
-        </is>
-      </c>
-      <c r="I79" t="inlineStr">
-        <is>
-          <t>ADM ISAIAS 01</t>
-        </is>
-      </c>
+          <t>(analítico não exportado)</t>
+        </is>
+      </c>
+      <c r="I79" t="inlineStr"/>
       <c r="J79" t="inlineStr"/>
       <c r="K79" t="n">
         <v>227.5</v>
@@ -6139,8 +6407,10 @@
           <t>21:17</t>
         </is>
       </c>
-      <c r="F80" t="n">
-        <v>44157</v>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>44157</t>
+        </is>
       </c>
       <c r="G80" t="inlineStr">
         <is>
@@ -6149,14 +6419,10 @@
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>MARIANA CHAVES</t>
-        </is>
-      </c>
-      <c r="I80" t="inlineStr">
-        <is>
-          <t>ADM ISAIAS 01</t>
-        </is>
-      </c>
+          <t>(analítico não exportado)</t>
+        </is>
+      </c>
+      <c r="I80" t="inlineStr"/>
       <c r="J80" t="inlineStr"/>
       <c r="K80" t="n">
         <v>138</v>
@@ -6209,8 +6475,10 @@
           <t>21:38</t>
         </is>
       </c>
-      <c r="F81" t="n">
-        <v>44163</v>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>44163</t>
+        </is>
       </c>
       <c r="G81" t="inlineStr">
         <is>
@@ -6219,14 +6487,10 @@
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>MARIANA CHAVES</t>
-        </is>
-      </c>
-      <c r="I81" t="inlineStr">
-        <is>
-          <t>ADM ISAIAS 01</t>
-        </is>
-      </c>
+          <t>(analítico não exportado)</t>
+        </is>
+      </c>
+      <c r="I81" t="inlineStr"/>
       <c r="J81" t="inlineStr"/>
       <c r="K81" t="n">
         <v>158.5</v>
@@ -6279,8 +6543,10 @@
           <t>21:44</t>
         </is>
       </c>
-      <c r="F82" t="n">
-        <v>44170</v>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>44170</t>
+        </is>
       </c>
       <c r="G82" t="inlineStr">
         <is>
@@ -6289,14 +6555,10 @@
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>MARIANA CHAVES</t>
-        </is>
-      </c>
-      <c r="I82" t="inlineStr">
-        <is>
-          <t>ADM ISAIAS 01</t>
-        </is>
-      </c>
+          <t>(analítico não exportado)</t>
+        </is>
+      </c>
+      <c r="I82" t="inlineStr"/>
       <c r="J82" t="inlineStr"/>
       <c r="K82" t="n">
         <v>212.5</v>
@@ -6349,8 +6611,10 @@
           <t>23:07</t>
         </is>
       </c>
-      <c r="F83" t="n">
-        <v>44220</v>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>44220</t>
+        </is>
       </c>
       <c r="G83" t="inlineStr">
         <is>
@@ -6359,14 +6623,10 @@
       </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t>MARIANA CHAVES</t>
-        </is>
-      </c>
-      <c r="I83" t="inlineStr">
-        <is>
-          <t>ADM ISAIAS 01</t>
-        </is>
-      </c>
+          <t>(analítico não exportado)</t>
+        </is>
+      </c>
+      <c r="I83" t="inlineStr"/>
       <c r="J83" t="inlineStr"/>
       <c r="K83" t="n">
         <v>117</v>
@@ -6533,8 +6793,10 @@
           <t>21:26</t>
         </is>
       </c>
-      <c r="F2" t="n">
-        <v>42146</v>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>42146</t>
+        </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -6599,8 +6861,10 @@
           <t>22:27</t>
         </is>
       </c>
-      <c r="F3" t="n">
-        <v>42162</v>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>42162</t>
+        </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
@@ -6665,8 +6929,10 @@
           <t>19:18</t>
         </is>
       </c>
-      <c r="F4" t="n">
-        <v>42685</v>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>42685</t>
+        </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
@@ -6731,8 +6997,10 @@
           <t>21:00</t>
         </is>
       </c>
-      <c r="F5" t="n">
-        <v>42689</v>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>42689</t>
+        </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
@@ -6797,8 +7065,10 @@
           <t>21:43</t>
         </is>
       </c>
-      <c r="F6" t="n">
-        <v>43112</v>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>43112</t>
+        </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
@@ -6863,8 +7133,10 @@
           <t>22:34</t>
         </is>
       </c>
-      <c r="F7" t="n">
-        <v>43125</v>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>43125</t>
+        </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
analítico de cupons das 17 lojas (01–19/10); ISAIAS taxa de serviço com operador completo
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015XeuzNyreGoe8Jd1wBUgeX
</commit_message>
<xml_diff>
--- a/saida/isaias_taxa_servico_2026-10-01_a_18.xlsx
+++ b/saida/isaias_taxa_servico_2026-10-01_a_18.xlsx
@@ -424,7 +424,7 @@
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
     <col width="21" customWidth="1" min="7" max="7"/>
-    <col width="27" customWidth="1" min="8" max="8"/>
+    <col width="23" customWidth="1" min="8" max="8"/>
     <col width="34" customWidth="1" min="9" max="9"/>
     <col width="10" customWidth="1" min="10" max="10"/>
     <col width="11" customWidth="1" min="11" max="11"/>
@@ -5875,11 +5875,19 @@
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>(analítico não exportado)</t>
-        </is>
-      </c>
-      <c r="I72" t="inlineStr"/>
-      <c r="J72" t="inlineStr"/>
+          <t>BRUNO DA SILVA INACIO</t>
+        </is>
+      </c>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DANIEL BACELAR XAVIER </t>
+        </is>
+      </c>
+      <c r="J72" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
       <c r="K72" t="n">
         <v>190</v>
       </c>
@@ -5943,11 +5951,19 @@
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>(analítico não exportado)</t>
-        </is>
-      </c>
-      <c r="I73" t="inlineStr"/>
-      <c r="J73" t="inlineStr"/>
+          <t>BRUNO DA SILVA INACIO</t>
+        </is>
+      </c>
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>DAVID FERNANDES DA CRUZ</t>
+        </is>
+      </c>
+      <c r="J73" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
       <c r="K73" t="n">
         <v>166.5</v>
       </c>
@@ -6011,11 +6027,19 @@
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>(analítico não exportado)</t>
-        </is>
-      </c>
-      <c r="I74" t="inlineStr"/>
-      <c r="J74" t="inlineStr"/>
+          <t>BRUNO DA SILVA INACIO</t>
+        </is>
+      </c>
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>MATEUS AUGUSTO NASCIMENTO COSTA</t>
+        </is>
+      </c>
+      <c r="J74" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
       <c r="K74" t="n">
         <v>342</v>
       </c>
@@ -6079,11 +6103,19 @@
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>(analítico não exportado)</t>
-        </is>
-      </c>
-      <c r="I75" t="inlineStr"/>
-      <c r="J75" t="inlineStr"/>
+          <t>BRUNO DA SILVA INACIO</t>
+        </is>
+      </c>
+      <c r="I75" t="inlineStr">
+        <is>
+          <t>DAVID FERNANDES DA CRUZ</t>
+        </is>
+      </c>
+      <c r="J75" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
       <c r="K75" t="n">
         <v>256</v>
       </c>
@@ -6147,11 +6179,19 @@
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>(analítico não exportado)</t>
-        </is>
-      </c>
-      <c r="I76" t="inlineStr"/>
-      <c r="J76" t="inlineStr"/>
+          <t>BRUNO DA SILVA INACIO</t>
+        </is>
+      </c>
+      <c r="I76" t="inlineStr">
+        <is>
+          <t>DAVID FERNANDES DA CRUZ</t>
+        </is>
+      </c>
+      <c r="J76" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
       <c r="K76" t="n">
         <v>103</v>
       </c>
@@ -6215,11 +6255,19 @@
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>(analítico não exportado)</t>
-        </is>
-      </c>
-      <c r="I77" t="inlineStr"/>
-      <c r="J77" t="inlineStr"/>
+          <t>BRUNO DA SILVA INACIO</t>
+        </is>
+      </c>
+      <c r="I77" t="inlineStr">
+        <is>
+          <t>MATEUS AUGUSTO NASCIMENTO COSTA</t>
+        </is>
+      </c>
+      <c r="J77" t="inlineStr">
+        <is>
+          <t>244</t>
+        </is>
+      </c>
       <c r="K77" t="n">
         <v>272</v>
       </c>
@@ -6283,11 +6331,19 @@
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>(analítico não exportado)</t>
-        </is>
-      </c>
-      <c r="I78" t="inlineStr"/>
-      <c r="J78" t="inlineStr"/>
+          <t>BRUNO DA SILVA INACIO</t>
+        </is>
+      </c>
+      <c r="I78" t="inlineStr">
+        <is>
+          <t>KEROLAINY LAWANY RIO BRANCO</t>
+        </is>
+      </c>
+      <c r="J78" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
       <c r="K78" t="n">
         <v>168</v>
       </c>
@@ -6351,11 +6407,19 @@
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>(analítico não exportado)</t>
-        </is>
-      </c>
-      <c r="I79" t="inlineStr"/>
-      <c r="J79" t="inlineStr"/>
+          <t>BRUNO DA SILVA INACIO</t>
+        </is>
+      </c>
+      <c r="I79" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DAIANA APARECIDA DOS SANTOS SILVA ALVES </t>
+        </is>
+      </c>
+      <c r="J79" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
       <c r="K79" t="n">
         <v>227.5</v>
       </c>
@@ -6419,11 +6483,19 @@
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>(analítico não exportado)</t>
-        </is>
-      </c>
-      <c r="I80" t="inlineStr"/>
-      <c r="J80" t="inlineStr"/>
+          <t>BRUNO DA SILVA INACIO</t>
+        </is>
+      </c>
+      <c r="I80" t="inlineStr">
+        <is>
+          <t>CAIO VINICIUS DOS SANTOS SILVA</t>
+        </is>
+      </c>
+      <c r="J80" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
       <c r="K80" t="n">
         <v>138</v>
       </c>
@@ -6487,11 +6559,19 @@
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>(analítico não exportado)</t>
-        </is>
-      </c>
-      <c r="I81" t="inlineStr"/>
-      <c r="J81" t="inlineStr"/>
+          <t>BRUNO DA SILVA INACIO</t>
+        </is>
+      </c>
+      <c r="I81" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DAIANA APARECIDA DOS SANTOS SILVA ALVES </t>
+        </is>
+      </c>
+      <c r="J81" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
       <c r="K81" t="n">
         <v>158.5</v>
       </c>
@@ -6555,11 +6635,19 @@
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>(analítico não exportado)</t>
-        </is>
-      </c>
-      <c r="I82" t="inlineStr"/>
-      <c r="J82" t="inlineStr"/>
+          <t>BRUNO DA SILVA INACIO</t>
+        </is>
+      </c>
+      <c r="I82" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DAIANA APARECIDA DOS SANTOS SILVA ALVES </t>
+        </is>
+      </c>
+      <c r="J82" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
       <c r="K82" t="n">
         <v>212.5</v>
       </c>
@@ -6623,11 +6711,19 @@
       </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t>(analítico não exportado)</t>
-        </is>
-      </c>
-      <c r="I83" t="inlineStr"/>
-      <c r="J83" t="inlineStr"/>
+          <t>BRUNO DA SILVA INACIO</t>
+        </is>
+      </c>
+      <c r="I83" t="inlineStr">
+        <is>
+          <t>DAVID FERNANDES DA CRUZ</t>
+        </is>
+      </c>
+      <c r="J83" t="inlineStr">
+        <is>
+          <t>227</t>
+        </is>
+      </c>
       <c r="K83" t="n">
         <v>117</v>
       </c>
@@ -6674,8 +6770,8 @@
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
     <col width="21" customWidth="1" min="7" max="7"/>
-    <col width="27" customWidth="1" min="8" max="8"/>
-    <col width="11" customWidth="1" min="9" max="9"/>
+    <col width="21" customWidth="1" min="8" max="8"/>
+    <col width="34" customWidth="1" min="9" max="9"/>
     <col width="10" customWidth="1" min="10" max="10"/>
     <col width="11" customWidth="1" min="11" max="11"/>
     <col width="15" customWidth="1" min="12" max="12"/>
@@ -6805,11 +6901,19 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>(analítico não exportado)</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr"/>
+          <t>PAULO CESAR BIANCHI</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>WILLIAN LUAN DANIEL FERREIRA DA SILVA</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
       <c r="K2" t="n">
         <v>379.5</v>
       </c>
@@ -6873,11 +6977,19 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>(analítico não exportado)</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr"/>
+          <t>PAULO CESAR BIANCHI</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>WELLINGTON GIAN DE JESUS</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
       <c r="K3" t="n">
         <v>90</v>
       </c>
@@ -6941,11 +7053,19 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>(analítico não exportado)</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr"/>
+          <t>PAULO CESAR BIANCHI</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>LUCIANO TEIXEIRA PEREIRA</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
       <c r="K4" t="n">
         <v>89</v>
       </c>
@@ -7009,11 +7129,19 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>(analítico não exportado)</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr"/>
+          <t>PAULO CESAR BIANCHI</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>LUCIANO TEIXEIRA PEREIRA</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="K5" t="n">
         <v>134</v>
       </c>
@@ -7077,11 +7205,19 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>(analítico não exportado)</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr"/>
-      <c r="J6" t="inlineStr"/>
+          <t>PAULO CESAR BIANCHI</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>WILLIAN LUAN DANIEL FERREIRA DA SILVA</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
       <c r="K6" t="n">
         <v>252.4</v>
       </c>
@@ -7145,11 +7281,19 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>(analítico não exportado)</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr"/>
-      <c r="J7" t="inlineStr"/>
+          <t>PAULO CESAR BIANCHI</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>WELLINGTON GIAN DE JESUS</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
       <c r="K7" t="n">
         <v>286</v>
       </c>

</xml_diff>

<commit_message>
ler_pdv/ler_tef: linha repetida dentro do mesmo arquivo é conta dividida e fica; só repetição entre arquivos sai
Corrige 146 cupons (R$ 8.020) com pagamentos iguais no mesmo cupom que estavam sendo apagados
desde a leitura multi-arquivo. Saídas e painel regerados.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015XeuzNyreGoe8Jd1wBUgeX
</commit_message>
<xml_diff>
--- a/saida/isaias_taxa_servico_2026-10-01_a_18.xlsx
+++ b/saida/isaias_taxa_servico_2026-10-01_a_18.xlsx
@@ -626,7 +626,7 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>PDV 02 em 106 de 106 casamentos exatos</t>
+          <t>PDV 02 em 108 de 108 casamentos exatos</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
@@ -726,7 +726,7 @@
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>PDV 02 em 106 de 106 casamentos exatos</t>
+          <t>PDV 02 em 108 de 108 casamentos exatos</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
@@ -826,7 +826,7 @@
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>PDV 02 em 106 de 106 casamentos exatos</t>
+          <t>PDV 02 em 108 de 108 casamentos exatos</t>
         </is>
       </c>
       <c r="R4" t="inlineStr">
@@ -926,7 +926,7 @@
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>PDV 02 em 106 de 106 casamentos exatos</t>
+          <t>PDV 02 em 108 de 108 casamentos exatos</t>
         </is>
       </c>
       <c r="R5" t="inlineStr">
@@ -1026,7 +1026,7 @@
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>PDV 02 em 106 de 106 casamentos exatos</t>
+          <t>PDV 02 em 108 de 108 casamentos exatos</t>
         </is>
       </c>
       <c r="R6" t="inlineStr">
@@ -1126,7 +1126,7 @@
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>PDV 02 em 106 de 106 casamentos exatos</t>
+          <t>PDV 02 em 108 de 108 casamentos exatos</t>
         </is>
       </c>
       <c r="R7" t="inlineStr">
@@ -1226,7 +1226,7 @@
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>PDV 02 em 106 de 106 casamentos exatos</t>
+          <t>PDV 02 em 108 de 108 casamentos exatos</t>
         </is>
       </c>
       <c r="R8" t="inlineStr">
@@ -1326,7 +1326,7 @@
       </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>PDV 02 em 128 de 128 casamentos exatos</t>
+          <t>PDV 02 em 131 de 131 casamentos exatos</t>
         </is>
       </c>
       <c r="R9" t="inlineStr">
@@ -1426,7 +1426,7 @@
       </c>
       <c r="Q10" t="inlineStr">
         <is>
-          <t>PDV 02 em 106 de 106 casamentos exatos</t>
+          <t>PDV 02 em 108 de 108 casamentos exatos</t>
         </is>
       </c>
       <c r="R10" t="inlineStr">
@@ -1526,7 +1526,7 @@
       </c>
       <c r="Q11" t="inlineStr">
         <is>
-          <t>PDV 02 em 128 de 128 casamentos exatos</t>
+          <t>PDV 02 em 131 de 131 casamentos exatos</t>
         </is>
       </c>
       <c r="R11" t="inlineStr">
@@ -1626,7 +1626,7 @@
       </c>
       <c r="Q12" t="inlineStr">
         <is>
-          <t>PDV 02 em 106 de 106 casamentos exatos</t>
+          <t>PDV 02 em 108 de 108 casamentos exatos</t>
         </is>
       </c>
       <c r="R12" t="inlineStr">
@@ -1726,7 +1726,7 @@
       </c>
       <c r="Q13" t="inlineStr">
         <is>
-          <t>PDV 02 em 128 de 128 casamentos exatos</t>
+          <t>PDV 02 em 131 de 131 casamentos exatos</t>
         </is>
       </c>
       <c r="R13" t="inlineStr">
@@ -1826,7 +1826,7 @@
       </c>
       <c r="Q14" t="inlineStr">
         <is>
-          <t>PDV 02 em 106 de 106 casamentos exatos</t>
+          <t>PDV 02 em 108 de 108 casamentos exatos</t>
         </is>
       </c>
       <c r="R14" t="inlineStr">
@@ -1926,7 +1926,7 @@
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>PDV 02 em 128 de 128 casamentos exatos</t>
+          <t>PDV 02 em 131 de 131 casamentos exatos</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
@@ -2026,7 +2026,7 @@
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>PDV 02 em 106 de 106 casamentos exatos</t>
+          <t>PDV 02 em 108 de 108 casamentos exatos</t>
         </is>
       </c>
       <c r="R16" t="inlineStr">
@@ -2126,7 +2126,7 @@
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>PDV 02 em 128 de 128 casamentos exatos</t>
+          <t>PDV 02 em 131 de 131 casamentos exatos</t>
         </is>
       </c>
       <c r="R17" t="inlineStr">
@@ -2226,7 +2226,7 @@
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>PDV 02 em 128 de 128 casamentos exatos</t>
+          <t>PDV 02 em 131 de 131 casamentos exatos</t>
         </is>
       </c>
       <c r="R18" t="inlineStr">
@@ -2326,7 +2326,7 @@
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>PDV 02 em 128 de 128 casamentos exatos</t>
+          <t>PDV 02 em 131 de 131 casamentos exatos</t>
         </is>
       </c>
       <c r="R19" t="inlineStr">
@@ -2426,7 +2426,7 @@
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>PDV 02 em 128 de 128 casamentos exatos</t>
+          <t>PDV 02 em 131 de 131 casamentos exatos</t>
         </is>
       </c>
       <c r="R20" t="inlineStr">
@@ -2526,7 +2526,7 @@
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>PDV 02 em 128 de 128 casamentos exatos</t>
+          <t>PDV 02 em 131 de 131 casamentos exatos</t>
         </is>
       </c>
       <c r="R21" t="inlineStr">
@@ -2626,7 +2626,7 @@
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>PDV 02 em 128 de 128 casamentos exatos</t>
+          <t>PDV 02 em 131 de 131 casamentos exatos</t>
         </is>
       </c>
       <c r="R22" t="inlineStr">
@@ -2726,7 +2726,7 @@
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>PDV 02 em 128 de 128 casamentos exatos</t>
+          <t>PDV 02 em 131 de 131 casamentos exatos</t>
         </is>
       </c>
       <c r="R23" t="inlineStr">
@@ -2826,7 +2826,7 @@
       </c>
       <c r="Q24" t="inlineStr">
         <is>
-          <t>PDV 02 em 106 de 106 casamentos exatos</t>
+          <t>PDV 02 em 108 de 108 casamentos exatos</t>
         </is>
       </c>
       <c r="R24" t="inlineStr">
@@ -2926,7 +2926,7 @@
       </c>
       <c r="Q25" t="inlineStr">
         <is>
-          <t>PDV 02 em 106 de 106 casamentos exatos</t>
+          <t>PDV 02 em 108 de 108 casamentos exatos</t>
         </is>
       </c>
       <c r="R25" t="inlineStr">
@@ -3026,7 +3026,7 @@
       </c>
       <c r="Q26" t="inlineStr">
         <is>
-          <t>PDV 02 em 106 de 106 casamentos exatos</t>
+          <t>PDV 02 em 108 de 108 casamentos exatos</t>
         </is>
       </c>
       <c r="R26" t="inlineStr">
@@ -3126,7 +3126,7 @@
       </c>
       <c r="Q27" t="inlineStr">
         <is>
-          <t>PDV 02 em 128 de 128 casamentos exatos</t>
+          <t>PDV 02 em 131 de 131 casamentos exatos</t>
         </is>
       </c>
       <c r="R27" t="inlineStr">
@@ -3226,7 +3226,7 @@
       </c>
       <c r="Q28" t="inlineStr">
         <is>
-          <t>PDV 02 em 128 de 128 casamentos exatos</t>
+          <t>PDV 02 em 131 de 131 casamentos exatos</t>
         </is>
       </c>
       <c r="R28" t="inlineStr">
@@ -3326,7 +3326,7 @@
       </c>
       <c r="Q29" t="inlineStr">
         <is>
-          <t>PDV 01 em 47 de 72 casamentos exatos</t>
+          <t>PDV 01 em 47 de 73 casamentos exatos</t>
         </is>
       </c>
       <c r="R29" t="inlineStr">
@@ -3426,7 +3426,7 @@
       </c>
       <c r="Q30" t="inlineStr">
         <is>
-          <t>PDV 02 em 106 de 106 casamentos exatos</t>
+          <t>PDV 02 em 108 de 108 casamentos exatos</t>
         </is>
       </c>
       <c r="R30" t="inlineStr">
@@ -3526,7 +3526,7 @@
       </c>
       <c r="Q31" t="inlineStr">
         <is>
-          <t>PDV 02 em 128 de 128 casamentos exatos</t>
+          <t>PDV 02 em 131 de 131 casamentos exatos</t>
         </is>
       </c>
       <c r="R31" t="inlineStr">
@@ -3626,7 +3626,7 @@
       </c>
       <c r="Q32" t="inlineStr">
         <is>
-          <t>PDV 02 em 128 de 128 casamentos exatos</t>
+          <t>PDV 02 em 131 de 131 casamentos exatos</t>
         </is>
       </c>
       <c r="R32" t="inlineStr">
@@ -3726,7 +3726,7 @@
       </c>
       <c r="Q33" t="inlineStr">
         <is>
-          <t>PDV 02 em 128 de 128 casamentos exatos</t>
+          <t>PDV 02 em 131 de 131 casamentos exatos</t>
         </is>
       </c>
       <c r="R33" t="inlineStr">
@@ -3826,7 +3826,7 @@
       </c>
       <c r="Q34" t="inlineStr">
         <is>
-          <t>PDV 02 em 128 de 128 casamentos exatos</t>
+          <t>PDV 02 em 131 de 131 casamentos exatos</t>
         </is>
       </c>
       <c r="R34" t="inlineStr">
@@ -3926,7 +3926,7 @@
       </c>
       <c r="Q35" t="inlineStr">
         <is>
-          <t>PDV 02 em 106 de 106 casamentos exatos</t>
+          <t>PDV 02 em 108 de 108 casamentos exatos</t>
         </is>
       </c>
       <c r="R35" t="inlineStr">
@@ -4026,7 +4026,7 @@
       </c>
       <c r="Q36" t="inlineStr">
         <is>
-          <t>PDV 02 em 106 de 106 casamentos exatos</t>
+          <t>PDV 02 em 108 de 108 casamentos exatos</t>
         </is>
       </c>
       <c r="R36" t="inlineStr">
@@ -4126,7 +4126,7 @@
       </c>
       <c r="Q37" t="inlineStr">
         <is>
-          <t>PDV 02 em 106 de 106 casamentos exatos</t>
+          <t>PDV 02 em 108 de 108 casamentos exatos</t>
         </is>
       </c>
       <c r="R37" t="inlineStr">
@@ -4226,7 +4226,7 @@
       </c>
       <c r="Q38" t="inlineStr">
         <is>
-          <t>PDV 02 em 128 de 128 casamentos exatos</t>
+          <t>PDV 02 em 131 de 131 casamentos exatos</t>
         </is>
       </c>
       <c r="R38" t="inlineStr">
@@ -4326,7 +4326,7 @@
       </c>
       <c r="Q39" t="inlineStr">
         <is>
-          <t>PDV 02 em 128 de 128 casamentos exatos</t>
+          <t>PDV 02 em 131 de 131 casamentos exatos</t>
         </is>
       </c>
       <c r="R39" t="inlineStr">
@@ -4426,7 +4426,7 @@
       </c>
       <c r="Q40" t="inlineStr">
         <is>
-          <t>PDV 02 em 106 de 106 casamentos exatos</t>
+          <t>PDV 02 em 108 de 108 casamentos exatos</t>
         </is>
       </c>
       <c r="R40" t="inlineStr">
@@ -4526,7 +4526,7 @@
       </c>
       <c r="Q41" t="inlineStr">
         <is>
-          <t>PDV 02 em 106 de 106 casamentos exatos</t>
+          <t>PDV 02 em 108 de 108 casamentos exatos</t>
         </is>
       </c>
       <c r="R41" t="inlineStr">
@@ -4626,7 +4626,7 @@
       </c>
       <c r="Q42" t="inlineStr">
         <is>
-          <t>PDV 02 em 106 de 106 casamentos exatos</t>
+          <t>PDV 02 em 108 de 108 casamentos exatos</t>
         </is>
       </c>
       <c r="R42" t="inlineStr">
@@ -4726,7 +4726,7 @@
       </c>
       <c r="Q43" t="inlineStr">
         <is>
-          <t>PDV 02 em 128 de 128 casamentos exatos</t>
+          <t>PDV 02 em 131 de 131 casamentos exatos</t>
         </is>
       </c>
       <c r="R43" t="inlineStr">
@@ -4826,7 +4826,7 @@
       </c>
       <c r="Q44" t="inlineStr">
         <is>
-          <t>PDV 02 em 106 de 106 casamentos exatos</t>
+          <t>PDV 02 em 108 de 108 casamentos exatos</t>
         </is>
       </c>
       <c r="R44" t="inlineStr">
@@ -4926,7 +4926,7 @@
       </c>
       <c r="Q45" t="inlineStr">
         <is>
-          <t>PDV 02 em 106 de 106 casamentos exatos</t>
+          <t>PDV 02 em 108 de 108 casamentos exatos</t>
         </is>
       </c>
       <c r="R45" t="inlineStr">
@@ -5026,7 +5026,7 @@
       </c>
       <c r="Q46" t="inlineStr">
         <is>
-          <t>PDV 02 em 106 de 106 casamentos exatos</t>
+          <t>PDV 02 em 108 de 108 casamentos exatos</t>
         </is>
       </c>
       <c r="R46" t="inlineStr">
@@ -5126,7 +5126,7 @@
       </c>
       <c r="Q47" t="inlineStr">
         <is>
-          <t>PDV 02 em 106 de 106 casamentos exatos</t>
+          <t>PDV 02 em 108 de 108 casamentos exatos</t>
         </is>
       </c>
       <c r="R47" t="inlineStr">
@@ -5226,7 +5226,7 @@
       </c>
       <c r="Q48" t="inlineStr">
         <is>
-          <t>PDV 02 em 106 de 106 casamentos exatos</t>
+          <t>PDV 02 em 108 de 108 casamentos exatos</t>
         </is>
       </c>
       <c r="R48" t="inlineStr">
@@ -5326,7 +5326,7 @@
       </c>
       <c r="Q49" t="inlineStr">
         <is>
-          <t>PDV 02 em 106 de 106 casamentos exatos</t>
+          <t>PDV 02 em 108 de 108 casamentos exatos</t>
         </is>
       </c>
       <c r="R49" t="inlineStr">
@@ -5426,7 +5426,7 @@
       </c>
       <c r="Q50" t="inlineStr">
         <is>
-          <t>PDV 02 em 106 de 106 casamentos exatos</t>
+          <t>PDV 02 em 108 de 108 casamentos exatos</t>
         </is>
       </c>
       <c r="R50" t="inlineStr">
@@ -5526,7 +5526,7 @@
       </c>
       <c r="Q51" t="inlineStr">
         <is>
-          <t>PDV 02 em 106 de 106 casamentos exatos</t>
+          <t>PDV 02 em 108 de 108 casamentos exatos</t>
         </is>
       </c>
       <c r="R51" t="inlineStr">
@@ -5626,7 +5626,7 @@
       </c>
       <c r="Q52" t="inlineStr">
         <is>
-          <t>PDV 02 em 128 de 128 casamentos exatos</t>
+          <t>PDV 02 em 131 de 131 casamentos exatos</t>
         </is>
       </c>
       <c r="R52" t="inlineStr">
@@ -5726,7 +5726,7 @@
       </c>
       <c r="Q53" t="inlineStr">
         <is>
-          <t>PDV 02 em 128 de 128 casamentos exatos</t>
+          <t>PDV 02 em 131 de 131 casamentos exatos</t>
         </is>
       </c>
       <c r="R53" t="inlineStr">
@@ -5826,7 +5826,7 @@
       </c>
       <c r="Q54" t="inlineStr">
         <is>
-          <t>PDV 02 em 128 de 128 casamentos exatos</t>
+          <t>PDV 02 em 131 de 131 casamentos exatos</t>
         </is>
       </c>
       <c r="R54" t="inlineStr">
@@ -5926,7 +5926,7 @@
       </c>
       <c r="Q55" t="inlineStr">
         <is>
-          <t>PDV 02 em 106 de 106 casamentos exatos</t>
+          <t>PDV 02 em 108 de 108 casamentos exatos</t>
         </is>
       </c>
       <c r="R55" t="inlineStr">
@@ -6026,7 +6026,7 @@
       </c>
       <c r="Q56" t="inlineStr">
         <is>
-          <t>PDV 02 em 128 de 128 casamentos exatos</t>
+          <t>PDV 02 em 131 de 131 casamentos exatos</t>
         </is>
       </c>
       <c r="R56" t="inlineStr">
@@ -6126,7 +6126,7 @@
       </c>
       <c r="Q57" t="inlineStr">
         <is>
-          <t>PDV 02 em 128 de 128 casamentos exatos</t>
+          <t>PDV 02 em 131 de 131 casamentos exatos</t>
         </is>
       </c>
       <c r="R57" t="inlineStr">
@@ -6226,7 +6226,7 @@
       </c>
       <c r="Q58" t="inlineStr">
         <is>
-          <t>PDV 02 em 128 de 128 casamentos exatos</t>
+          <t>PDV 02 em 131 de 131 casamentos exatos</t>
         </is>
       </c>
       <c r="R58" t="inlineStr">
@@ -6326,7 +6326,7 @@
       </c>
       <c r="Q59" t="inlineStr">
         <is>
-          <t>PDV 02 em 106 de 106 casamentos exatos</t>
+          <t>PDV 02 em 108 de 108 casamentos exatos</t>
         </is>
       </c>
       <c r="R59" t="inlineStr">
@@ -6426,7 +6426,7 @@
       </c>
       <c r="Q60" t="inlineStr">
         <is>
-          <t>PDV 02 em 106 de 106 casamentos exatos</t>
+          <t>PDV 02 em 108 de 108 casamentos exatos</t>
         </is>
       </c>
       <c r="R60" t="inlineStr">
@@ -6526,7 +6526,7 @@
       </c>
       <c r="Q61" t="inlineStr">
         <is>
-          <t>PDV 02 em 106 de 106 casamentos exatos</t>
+          <t>PDV 02 em 108 de 108 casamentos exatos</t>
         </is>
       </c>
       <c r="R61" t="inlineStr">
@@ -6626,7 +6626,7 @@
       </c>
       <c r="Q62" t="inlineStr">
         <is>
-          <t>PDV 02 em 128 de 128 casamentos exatos</t>
+          <t>PDV 02 em 131 de 131 casamentos exatos</t>
         </is>
       </c>
       <c r="R62" t="inlineStr">
@@ -6726,7 +6726,7 @@
       </c>
       <c r="Q63" t="inlineStr">
         <is>
-          <t>PDV 02 em 128 de 128 casamentos exatos</t>
+          <t>PDV 02 em 131 de 131 casamentos exatos</t>
         </is>
       </c>
       <c r="R63" t="inlineStr">
@@ -6826,7 +6826,7 @@
       </c>
       <c r="Q64" t="inlineStr">
         <is>
-          <t>PDV 02 em 128 de 128 casamentos exatos</t>
+          <t>PDV 02 em 131 de 131 casamentos exatos</t>
         </is>
       </c>
       <c r="R64" t="inlineStr">
@@ -6926,7 +6926,7 @@
       </c>
       <c r="Q65" t="inlineStr">
         <is>
-          <t>PDV 02 em 128 de 128 casamentos exatos</t>
+          <t>PDV 02 em 131 de 131 casamentos exatos</t>
         </is>
       </c>
       <c r="R65" t="inlineStr">
@@ -7026,7 +7026,7 @@
       </c>
       <c r="Q66" t="inlineStr">
         <is>
-          <t>PDV 02 em 128 de 128 casamentos exatos</t>
+          <t>PDV 02 em 131 de 131 casamentos exatos</t>
         </is>
       </c>
       <c r="R66" t="inlineStr">
@@ -7126,7 +7126,7 @@
       </c>
       <c r="Q67" t="inlineStr">
         <is>
-          <t>PDV 02 em 128 de 128 casamentos exatos</t>
+          <t>PDV 02 em 131 de 131 casamentos exatos</t>
         </is>
       </c>
       <c r="R67" t="inlineStr">
@@ -7226,7 +7226,7 @@
       </c>
       <c r="Q68" t="inlineStr">
         <is>
-          <t>PDV 02 em 128 de 128 casamentos exatos</t>
+          <t>PDV 02 em 131 de 131 casamentos exatos</t>
         </is>
       </c>
       <c r="R68" t="inlineStr">
@@ -7326,7 +7326,7 @@
       </c>
       <c r="Q69" t="inlineStr">
         <is>
-          <t>PDV 02 em 128 de 128 casamentos exatos</t>
+          <t>PDV 02 em 131 de 131 casamentos exatos</t>
         </is>
       </c>
       <c r="R69" t="inlineStr">
@@ -7426,7 +7426,7 @@
       </c>
       <c r="Q70" t="inlineStr">
         <is>
-          <t>PDV 02 em 128 de 128 casamentos exatos</t>
+          <t>PDV 02 em 131 de 131 casamentos exatos</t>
         </is>
       </c>
       <c r="R70" t="inlineStr">
@@ -7526,7 +7526,7 @@
       </c>
       <c r="Q71" t="inlineStr">
         <is>
-          <t>PDV 02 em 128 de 128 casamentos exatos</t>
+          <t>PDV 02 em 131 de 131 casamentos exatos</t>
         </is>
       </c>
       <c r="R71" t="inlineStr">
@@ -7626,7 +7626,7 @@
       </c>
       <c r="Q72" t="inlineStr">
         <is>
-          <t>PDV 02 em 128 de 128 casamentos exatos</t>
+          <t>PDV 02 em 131 de 131 casamentos exatos</t>
         </is>
       </c>
       <c r="R72" t="inlineStr">
@@ -7726,7 +7726,7 @@
       </c>
       <c r="Q73" t="inlineStr">
         <is>
-          <t>PDV 02 em 128 de 128 casamentos exatos</t>
+          <t>PDV 02 em 131 de 131 casamentos exatos</t>
         </is>
       </c>
       <c r="R73" t="inlineStr">
@@ -7826,7 +7826,7 @@
       </c>
       <c r="Q74" t="inlineStr">
         <is>
-          <t>PDV 02 em 106 de 106 casamentos exatos</t>
+          <t>PDV 02 em 108 de 108 casamentos exatos</t>
         </is>
       </c>
       <c r="R74" t="inlineStr">
@@ -7926,7 +7926,7 @@
       </c>
       <c r="Q75" t="inlineStr">
         <is>
-          <t>PDV 02 em 106 de 106 casamentos exatos</t>
+          <t>PDV 02 em 108 de 108 casamentos exatos</t>
         </is>
       </c>
       <c r="R75" t="inlineStr">
@@ -8026,7 +8026,7 @@
       </c>
       <c r="Q76" t="inlineStr">
         <is>
-          <t>PDV 02 em 106 de 106 casamentos exatos</t>
+          <t>PDV 02 em 108 de 108 casamentos exatos</t>
         </is>
       </c>
       <c r="R76" t="inlineStr">
@@ -8126,7 +8126,7 @@
       </c>
       <c r="Q77" t="inlineStr">
         <is>
-          <t>PDV 02 em 106 de 106 casamentos exatos</t>
+          <t>PDV 02 em 108 de 108 casamentos exatos</t>
         </is>
       </c>
       <c r="R77" t="inlineStr">
@@ -8226,7 +8226,7 @@
       </c>
       <c r="Q78" t="inlineStr">
         <is>
-          <t>PDV 02 em 128 de 128 casamentos exatos</t>
+          <t>PDV 02 em 131 de 131 casamentos exatos</t>
         </is>
       </c>
       <c r="R78" t="inlineStr">
@@ -8326,7 +8326,7 @@
       </c>
       <c r="Q79" t="inlineStr">
         <is>
-          <t>PDV 02 em 128 de 128 casamentos exatos</t>
+          <t>PDV 02 em 131 de 131 casamentos exatos</t>
         </is>
       </c>
       <c r="R79" t="inlineStr">
@@ -8426,7 +8426,7 @@
       </c>
       <c r="Q80" t="inlineStr">
         <is>
-          <t>PDV 02 em 128 de 128 casamentos exatos</t>
+          <t>PDV 02 em 131 de 131 casamentos exatos</t>
         </is>
       </c>
       <c r="R80" t="inlineStr">
@@ -8526,7 +8526,7 @@
       </c>
       <c r="Q81" t="inlineStr">
         <is>
-          <t>PDV 02 em 128 de 128 casamentos exatos</t>
+          <t>PDV 02 em 131 de 131 casamentos exatos</t>
         </is>
       </c>
       <c r="R81" t="inlineStr">
@@ -8626,7 +8626,7 @@
       </c>
       <c r="Q82" t="inlineStr">
         <is>
-          <t>PDV 02 em 128 de 128 casamentos exatos</t>
+          <t>PDV 02 em 131 de 131 casamentos exatos</t>
         </is>
       </c>
       <c r="R82" t="inlineStr">
@@ -8726,7 +8726,7 @@
       </c>
       <c r="Q83" t="inlineStr">
         <is>
-          <t>PDV 02 em 128 de 128 casamentos exatos</t>
+          <t>PDV 02 em 131 de 131 casamentos exatos</t>
         </is>
       </c>
       <c r="R83" t="inlineStr">
@@ -8976,7 +8976,7 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>PDV 01 em 167 de 167 casamentos exatos</t>
+          <t>PDV 01 em 168 de 168 casamentos exatos</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
@@ -9076,7 +9076,7 @@
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>PDV 01 em 167 de 167 casamentos exatos</t>
+          <t>PDV 01 em 168 de 168 casamentos exatos</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
@@ -9276,7 +9276,7 @@
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>PDV 01 em 167 de 167 casamentos exatos</t>
+          <t>PDV 01 em 168 de 168 casamentos exatos</t>
         </is>
       </c>
       <c r="R5" t="inlineStr">
@@ -9376,7 +9376,7 @@
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>PDV 01 em 124 de 124 casamentos exatos</t>
+          <t>PDV 01 em 127 de 127 casamentos exatos</t>
         </is>
       </c>
       <c r="R6" t="inlineStr">
@@ -9476,7 +9476,7 @@
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>PDV 01 em 167 de 167 casamentos exatos</t>
+          <t>PDV 01 em 168 de 168 casamentos exatos</t>
         </is>
       </c>
       <c r="R7" t="inlineStr">

</xml_diff>